<commit_message>
Add new files for orientation details and update existing resources
</commit_message>
<xml_diff>
--- a/Students Details.xlsx
+++ b/Students Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Krishnendu.Jana\Desktop\MITVPU-Orientation-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFF2DF73-E74B-4FC9-AAAA-C1A32CBE6956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F588060-261B-449B-88E9-8CC8A3ADB0F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7991DB97-C80E-432A-B6FF-7E61A06C8A94}"/>
   </bookViews>
@@ -4806,6 +4806,9 @@
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A162">
+        <v>161</v>
+      </c>
       <c r="B162" t="s">
         <v>336</v>
       </c>
@@ -4820,6 +4823,9 @@
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A163">
+        <v>162</v>
+      </c>
       <c r="B163" t="s">
         <v>338</v>
       </c>
@@ -4834,6 +4840,9 @@
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A164">
+        <v>163</v>
+      </c>
       <c r="B164" t="s">
         <v>340</v>
       </c>
@@ -4848,6 +4857,9 @@
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A165">
+        <v>164</v>
+      </c>
       <c r="B165" t="s">
         <v>342</v>
       </c>
@@ -4862,6 +4874,9 @@
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A166">
+        <v>165</v>
+      </c>
       <c r="B166" t="s">
         <v>344</v>
       </c>
@@ -4876,6 +4891,9 @@
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A167">
+        <v>166</v>
+      </c>
       <c r="B167" t="s">
         <v>346</v>
       </c>
@@ -4890,6 +4908,9 @@
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A168">
+        <v>167</v>
+      </c>
       <c r="B168" t="s">
         <v>348</v>
       </c>
@@ -4904,6 +4925,9 @@
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A169">
+        <v>168</v>
+      </c>
       <c r="B169" t="s">
         <v>352</v>
       </c>
@@ -4918,6 +4942,9 @@
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A170">
+        <v>169</v>
+      </c>
       <c r="B170" t="s">
         <v>354</v>
       </c>
@@ -4932,6 +4959,9 @@
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A171">
+        <v>170</v>
+      </c>
       <c r="B171" t="s">
         <v>356</v>
       </c>
@@ -4946,6 +4976,9 @@
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A172">
+        <v>171</v>
+      </c>
       <c r="B172" t="s">
         <v>358</v>
       </c>
@@ -4960,6 +4993,9 @@
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A173">
+        <v>172</v>
+      </c>
       <c r="B173" t="s">
         <v>360</v>
       </c>
@@ -4974,6 +5010,9 @@
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A174">
+        <v>173</v>
+      </c>
       <c r="B174" t="s">
         <v>362</v>
       </c>
@@ -4988,6 +5027,9 @@
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A175">
+        <v>174</v>
+      </c>
       <c r="B175" t="s">
         <v>364</v>
       </c>
@@ -5002,6 +5044,9 @@
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A176">
+        <v>175</v>
+      </c>
       <c r="B176" t="s">
         <v>366</v>
       </c>
@@ -5015,7 +5060,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="177" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A177">
+        <v>176</v>
+      </c>
       <c r="B177" t="s">
         <v>368</v>
       </c>
@@ -5029,7 +5077,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="178" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A178">
+        <v>177</v>
+      </c>
       <c r="B178" t="s">
         <v>370</v>
       </c>
@@ -5043,7 +5094,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="179" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A179">
+        <v>178</v>
+      </c>
       <c r="B179" t="s">
         <v>372</v>
       </c>
@@ -5057,7 +5111,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="180" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A180">
+        <v>179</v>
+      </c>
       <c r="B180" t="s">
         <v>374</v>
       </c>
@@ -5071,7 +5128,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="181" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A181">
+        <v>180</v>
+      </c>
       <c r="B181" t="s">
         <v>376</v>
       </c>
@@ -5085,7 +5145,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="182" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A182">
+        <v>181</v>
+      </c>
       <c r="B182" t="s">
         <v>378</v>
       </c>
@@ -5099,7 +5162,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="183" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A183">
+        <v>182</v>
+      </c>
       <c r="B183" t="s">
         <v>380</v>
       </c>
@@ -5113,7 +5179,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="184" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A184">
+        <v>183</v>
+      </c>
       <c r="B184" t="s">
         <v>382</v>
       </c>
@@ -5127,7 +5196,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="185" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A185">
+        <v>184</v>
+      </c>
       <c r="B185" t="s">
         <v>384</v>
       </c>
@@ -5141,7 +5213,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="186" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A186">
+        <v>185</v>
+      </c>
       <c r="B186" t="s">
         <v>386</v>
       </c>
@@ -5155,7 +5230,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="187" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A187">
+        <v>186</v>
+      </c>
       <c r="B187" t="s">
         <v>388</v>
       </c>
@@ -5169,7 +5247,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="188" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A188">
+        <v>187</v>
+      </c>
       <c r="B188" t="s">
         <v>390</v>
       </c>
@@ -5183,7 +5264,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="189" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A189">
+        <v>188</v>
+      </c>
       <c r="B189" t="s">
         <v>392</v>
       </c>
@@ -5197,7 +5281,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="190" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A190">
+        <v>189</v>
+      </c>
       <c r="B190" t="s">
         <v>394</v>
       </c>
@@ -5211,7 +5298,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="191" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A191">
+        <v>190</v>
+      </c>
       <c r="B191" t="s">
         <v>396</v>
       </c>
@@ -5225,7 +5315,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="192" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A192">
+        <v>191</v>
+      </c>
       <c r="B192" t="s">
         <v>398</v>
       </c>
@@ -5239,7 +5332,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="193" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A193">
+        <v>192</v>
+      </c>
       <c r="B193" t="s">
         <v>400</v>
       </c>
@@ -5253,7 +5349,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="194" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A194">
+        <v>193</v>
+      </c>
       <c r="B194" t="s">
         <v>402</v>
       </c>
@@ -5267,7 +5366,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="195" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A195">
+        <v>194</v>
+      </c>
       <c r="B195" t="s">
         <v>404</v>
       </c>
@@ -5281,7 +5383,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="196" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A196">
+        <v>195</v>
+      </c>
       <c r="B196" t="s">
         <v>406</v>
       </c>
@@ -5295,7 +5400,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="197" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A197">
+        <v>196</v>
+      </c>
       <c r="B197" t="s">
         <v>408</v>
       </c>
@@ -5309,7 +5417,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="198" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A198">
+        <v>197</v>
+      </c>
       <c r="B198" t="s">
         <v>410</v>
       </c>
@@ -5323,7 +5434,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="199" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A199">
+        <v>198</v>
+      </c>
       <c r="B199" t="s">
         <v>412</v>
       </c>
@@ -5337,7 +5451,10 @@
         <v>351</v>
       </c>
     </row>
-    <row r="200" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A200">
+        <v>199</v>
+      </c>
       <c r="B200" t="s">
         <v>414</v>
       </c>
@@ -5351,7 +5468,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="201" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A201">
+        <v>200</v>
+      </c>
       <c r="B201" t="s">
         <v>417</v>
       </c>
@@ -5365,7 +5485,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="202" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A202">
+        <v>201</v>
+      </c>
       <c r="B202" t="s">
         <v>419</v>
       </c>
@@ -5379,7 +5502,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="203" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A203">
+        <v>202</v>
+      </c>
       <c r="B203" t="s">
         <v>421</v>
       </c>
@@ -5393,7 +5519,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="204" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A204">
+        <v>203</v>
+      </c>
       <c r="B204" t="s">
         <v>423</v>
       </c>
@@ -5407,7 +5536,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="205" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A205">
+        <v>204</v>
+      </c>
       <c r="B205" t="s">
         <v>425</v>
       </c>
@@ -5421,7 +5553,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="206" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A206">
+        <v>205</v>
+      </c>
       <c r="B206" t="s">
         <v>427</v>
       </c>
@@ -5435,7 +5570,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="207" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A207">
+        <v>206</v>
+      </c>
       <c r="B207" t="s">
         <v>429</v>
       </c>
@@ -5449,7 +5587,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="208" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A208">
+        <v>207</v>
+      </c>
       <c r="B208" t="s">
         <v>431</v>
       </c>
@@ -5463,7 +5604,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="209" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A209">
+        <v>208</v>
+      </c>
       <c r="B209" t="s">
         <v>433</v>
       </c>
@@ -5477,7 +5621,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="210" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A210">
+        <v>209</v>
+      </c>
       <c r="B210" t="s">
         <v>435</v>
       </c>
@@ -5491,7 +5638,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="211" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A211">
+        <v>210</v>
+      </c>
       <c r="B211" t="s">
         <v>437</v>
       </c>
@@ -5505,7 +5655,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="212" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A212">
+        <v>211</v>
+      </c>
       <c r="B212" t="s">
         <v>439</v>
       </c>
@@ -5519,7 +5672,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="213" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A213">
+        <v>212</v>
+      </c>
       <c r="B213" t="s">
         <v>441</v>
       </c>
@@ -5533,7 +5689,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="214" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A214">
+        <v>213</v>
+      </c>
       <c r="B214" t="s">
         <v>444</v>
       </c>
@@ -5547,7 +5706,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="215" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A215">
+        <v>214</v>
+      </c>
       <c r="B215" t="s">
         <v>446</v>
       </c>
@@ -5561,7 +5723,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="216" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A216">
+        <v>215</v>
+      </c>
       <c r="B216" t="s">
         <v>448</v>
       </c>
@@ -5575,7 +5740,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="217" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A217">
+        <v>216</v>
+      </c>
       <c r="B217" t="s">
         <v>450</v>
       </c>
@@ -5589,7 +5757,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="218" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A218">
+        <v>217</v>
+      </c>
       <c r="B218" t="s">
         <v>452</v>
       </c>
@@ -5603,7 +5774,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="219" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A219">
+        <v>218</v>
+      </c>
       <c r="B219" t="s">
         <v>454</v>
       </c>
@@ -5617,7 +5791,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="220" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A220">
+        <v>219</v>
+      </c>
       <c r="B220" t="s">
         <v>456</v>
       </c>
@@ -5631,7 +5808,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="221" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A221">
+        <v>220</v>
+      </c>
       <c r="B221" t="s">
         <v>458</v>
       </c>
@@ -5645,7 +5825,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="222" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A222">
+        <v>221</v>
+      </c>
       <c r="B222" t="s">
         <v>460</v>
       </c>
@@ -5659,7 +5842,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="223" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A223">
+        <v>222</v>
+      </c>
       <c r="B223" t="s">
         <v>462</v>
       </c>
@@ -5673,7 +5859,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="224" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A224">
+        <v>223</v>
+      </c>
       <c r="B224" t="s">
         <v>464</v>
       </c>
@@ -5687,7 +5876,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="225" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A225">
+        <v>224</v>
+      </c>
       <c r="B225" t="s">
         <v>466</v>
       </c>
@@ -5701,7 +5893,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="226" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A226">
+        <v>225</v>
+      </c>
       <c r="B226" t="s">
         <v>469</v>
       </c>
@@ -5715,7 +5910,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="227" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A227">
+        <v>226</v>
+      </c>
       <c r="B227" t="s">
         <v>471</v>
       </c>
@@ -5729,7 +5927,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="228" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A228">
+        <v>227</v>
+      </c>
       <c r="B228" t="s">
         <v>473</v>
       </c>
@@ -5743,7 +5944,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="229" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A229">
+        <v>228</v>
+      </c>
       <c r="B229" t="s">
         <v>475</v>
       </c>
@@ -5757,7 +5961,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="230" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A230">
+        <v>229</v>
+      </c>
       <c r="B230" t="s">
         <v>477</v>
       </c>
@@ -5771,7 +5978,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="231" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A231">
+        <v>230</v>
+      </c>
       <c r="B231" t="s">
         <v>479</v>
       </c>
@@ -5785,7 +5995,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="232" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A232">
+        <v>231</v>
+      </c>
       <c r="B232" t="s">
         <v>481</v>
       </c>
@@ -5799,7 +6012,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="233" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A233">
+        <v>232</v>
+      </c>
       <c r="B233" t="s">
         <v>483</v>
       </c>
@@ -5813,7 +6029,10 @@
         <v>416</v>
       </c>
     </row>
-    <row r="234" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A234">
+        <v>233</v>
+      </c>
       <c r="B234" t="s">
         <v>485</v>
       </c>
@@ -5827,7 +6046,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="235" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A235">
+        <v>234</v>
+      </c>
       <c r="B235" t="s">
         <v>489</v>
       </c>
@@ -5841,7 +6063,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="236" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A236">
+        <v>235</v>
+      </c>
       <c r="B236" t="s">
         <v>491</v>
       </c>
@@ -5855,7 +6080,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="237" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A237">
+        <v>236</v>
+      </c>
       <c r="B237" t="s">
         <v>493</v>
       </c>
@@ -5869,7 +6097,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="238" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A238">
+        <v>237</v>
+      </c>
       <c r="B238" t="s">
         <v>495</v>
       </c>
@@ -5883,7 +6114,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="239" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A239">
+        <v>238</v>
+      </c>
       <c r="B239" t="s">
         <v>497</v>
       </c>
@@ -5897,7 +6131,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="240" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A240">
+        <v>239</v>
+      </c>
       <c r="B240" t="s">
         <v>499</v>
       </c>
@@ -5911,7 +6148,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="241" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A241">
+        <v>240</v>
+      </c>
       <c r="B241" t="s">
         <v>501</v>
       </c>
@@ -5925,7 +6165,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="242" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A242">
+        <v>241</v>
+      </c>
       <c r="B242" t="s">
         <v>503</v>
       </c>
@@ -5939,7 +6182,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="243" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A243">
+        <v>242</v>
+      </c>
       <c r="B243" t="s">
         <v>505</v>
       </c>
@@ -5953,7 +6199,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="244" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A244">
+        <v>243</v>
+      </c>
       <c r="B244" t="s">
         <v>507</v>
       </c>
@@ -5967,7 +6216,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="245" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A245">
+        <v>244</v>
+      </c>
       <c r="B245" t="s">
         <v>510</v>
       </c>
@@ -5981,7 +6233,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="246" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A246">
+        <v>245</v>
+      </c>
       <c r="B246" t="s">
         <v>512</v>
       </c>
@@ -5995,7 +6250,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="247" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A247">
+        <v>246</v>
+      </c>
       <c r="B247" t="s">
         <v>515</v>
       </c>
@@ -6009,7 +6267,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="248" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A248">
+        <v>247</v>
+      </c>
       <c r="B248" t="s">
         <v>517</v>
       </c>
@@ -6023,7 +6284,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="249" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A249">
+        <v>248</v>
+      </c>
       <c r="B249" t="s">
         <v>519</v>
       </c>
@@ -6037,7 +6301,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="250" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A250">
+        <v>249</v>
+      </c>
       <c r="B250" t="s">
         <v>522</v>
       </c>
@@ -6051,7 +6318,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="251" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A251">
+        <v>250</v>
+      </c>
       <c r="B251" t="s">
         <v>524</v>
       </c>
@@ -6065,7 +6335,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="252" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A252">
+        <v>251</v>
+      </c>
       <c r="B252" t="s">
         <v>527</v>
       </c>
@@ -6079,7 +6352,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="253" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A253">
+        <v>252</v>
+      </c>
       <c r="B253" t="s">
         <v>529</v>
       </c>
@@ -6093,7 +6369,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="254" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A254">
+        <v>253</v>
+      </c>
       <c r="B254" t="s">
         <v>531</v>
       </c>
@@ -6107,7 +6386,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="255" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A255">
+        <v>254</v>
+      </c>
       <c r="B255" t="s">
         <v>533</v>
       </c>
@@ -6121,7 +6403,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="256" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A256">
+        <v>255</v>
+      </c>
       <c r="B256" t="s">
         <v>535</v>
       </c>
@@ -6135,7 +6420,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="257" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A257">
+        <v>256</v>
+      </c>
       <c r="B257" t="s">
         <v>537</v>
       </c>
@@ -6149,7 +6437,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="258" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A258">
+        <v>257</v>
+      </c>
       <c r="B258" t="s">
         <v>539</v>
       </c>
@@ -6163,7 +6454,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="259" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A259">
+        <v>258</v>
+      </c>
       <c r="B259" t="s">
         <v>541</v>
       </c>
@@ -6177,7 +6471,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="260" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A260">
+        <v>259</v>
+      </c>
       <c r="B260" t="s">
         <v>544</v>
       </c>
@@ -6191,7 +6488,10 @@
         <v>488</v>
       </c>
     </row>
-    <row r="261" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A261">
+        <v>260</v>
+      </c>
       <c r="B261" t="s">
         <v>546</v>
       </c>

</xml_diff>

<commit_message>
Update roster and add missing B. Pharm. LE room mapping
Regenerate data.js from the latest Students Details.xlsx (new
students across several programs, now 275 total). The refreshed
roster introduced a "B. Pharm. LE" program with no registration room
mapping, which generate_data.py's own warning caught; mapped it to
the same room as B.Pharm (Room 517 / 518, School of Pharmacy).
</commit_message>
<xml_diff>
--- a/Students Details.xlsx
+++ b/Students Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Krishnendu.Jana\Desktop\MITVPU-Orientation-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F588060-261B-449B-88E9-8CC8A3ADB0F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E534BB-9B99-4F64-A8DB-EC9227FAD183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7991DB97-C80E-432A-B6FF-7E61A06C8A94}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1045" uniqueCount="548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="579">
   <si>
     <t>PRN</t>
   </si>
@@ -1683,6 +1683,99 @@
   </si>
   <si>
     <t>Yerwa Shrutika Avinash</t>
+  </si>
+  <si>
+    <t>SCFU426024</t>
+  </si>
+  <si>
+    <t>Hasan Ahmed Abraar Ahmed Shaikh</t>
+  </si>
+  <si>
+    <t>SEFU126010</t>
+  </si>
+  <si>
+    <t>Bomane Suyash Shivling</t>
+  </si>
+  <si>
+    <t>SEFU126011</t>
+  </si>
+  <si>
+    <t>Kharade Sarthak Dasharath</t>
+  </si>
+  <si>
+    <t>SEFU126012</t>
+  </si>
+  <si>
+    <t>Hulle Aadesh Abhay</t>
+  </si>
+  <si>
+    <t>SCFU126039</t>
+  </si>
+  <si>
+    <t>Thorat Soniya Satishkumar</t>
+  </si>
+  <si>
+    <t>SCLU326040</t>
+  </si>
+  <si>
+    <t>Kassa Siddharth Omprakash</t>
+  </si>
+  <si>
+    <t>SCFP126058</t>
+  </si>
+  <si>
+    <t>Motgi  Varad Vivek</t>
+  </si>
+  <si>
+    <t>SCFU226011</t>
+  </si>
+  <si>
+    <t>Bipeen Santosh Patil</t>
+  </si>
+  <si>
+    <t>BSFP226011</t>
+  </si>
+  <si>
+    <t>Ghiware Vinayak Shiwanand</t>
+  </si>
+  <si>
+    <t>BSFP226012</t>
+  </si>
+  <si>
+    <t>Chougule Pratik Sanjay</t>
+  </si>
+  <si>
+    <t>SDFU226003</t>
+  </si>
+  <si>
+    <t>Holikatti Apoorva Subhashchandra</t>
+  </si>
+  <si>
+    <t>SDFU226004</t>
+  </si>
+  <si>
+    <t>Rida Muzaffarhusain Maniyar</t>
+  </si>
+  <si>
+    <t>BSFU126046</t>
+  </si>
+  <si>
+    <t>Jagirdar Sadaf Moin</t>
+  </si>
+  <si>
+    <t>BSFP126010</t>
+  </si>
+  <si>
+    <t>Ambarkar Jai Girish</t>
+  </si>
+  <si>
+    <t>SPLU126001</t>
+  </si>
+  <si>
+    <t>Sujal Sanjay Banarjee</t>
+  </si>
+  <si>
+    <t>B. Pharm. LE</t>
   </si>
 </sst>
 </file>
@@ -2060,7 +2153,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81D7E270-40BB-453E-AA25-D300316939A2}">
-  <dimension ref="A1:E261"/>
+  <dimension ref="A1:E276"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
@@ -3076,13 +3169,13 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>129</v>
+        <v>548</v>
       </c>
       <c r="C60" t="s">
-        <v>130</v>
+        <v>549</v>
       </c>
       <c r="D60" t="s">
-        <v>131</v>
+        <v>84</v>
       </c>
       <c r="E60" t="s">
         <v>8</v>
@@ -3093,10 +3186,10 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C61" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D61" t="s">
         <v>131</v>
@@ -3110,10 +3203,10 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C62" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D62" t="s">
         <v>131</v>
@@ -3127,10 +3220,10 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C63" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D63" t="s">
         <v>131</v>
@@ -3144,10 +3237,10 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C64" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D64" t="s">
         <v>131</v>
@@ -3161,10 +3254,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C65" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D65" t="s">
         <v>131</v>
@@ -3178,10 +3271,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C66" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D66" t="s">
         <v>131</v>
@@ -3195,10 +3288,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C67" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D67" t="s">
         <v>131</v>
@@ -3212,10 +3305,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C68" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D68" t="s">
         <v>131</v>
@@ -3229,16 +3322,16 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C69" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D69" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="E69" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
@@ -3246,16 +3339,16 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>151</v>
+        <v>550</v>
       </c>
       <c r="C70" t="s">
-        <v>152</v>
+        <v>551</v>
       </c>
       <c r="D70" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="E70" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
@@ -3263,16 +3356,16 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>153</v>
+        <v>552</v>
       </c>
       <c r="C71" t="s">
-        <v>154</v>
+        <v>553</v>
       </c>
       <c r="D71" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="E71" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
@@ -3280,16 +3373,16 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>155</v>
+        <v>554</v>
       </c>
       <c r="C72" t="s">
-        <v>156</v>
+        <v>555</v>
       </c>
       <c r="D72" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="E72" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
@@ -3297,10 +3390,10 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="C73" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="D73" t="s">
         <v>150</v>
@@ -3314,10 +3407,10 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C74" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="D74" t="s">
         <v>150</v>
@@ -3331,10 +3424,10 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="C75" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D75" t="s">
         <v>150</v>
@@ -3348,10 +3441,10 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="C76" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="D76" t="s">
         <v>150</v>
@@ -3365,10 +3458,10 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="C77" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="D77" t="s">
         <v>150</v>
@@ -3382,10 +3475,10 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C78" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D78" t="s">
         <v>150</v>
@@ -3399,10 +3492,10 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="C79" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="D79" t="s">
         <v>150</v>
@@ -3416,10 +3509,10 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="C80" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D80" t="s">
         <v>150</v>
@@ -3433,10 +3526,10 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="C81" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="D81" t="s">
         <v>150</v>
@@ -3450,10 +3543,10 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="C82" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="D82" t="s">
         <v>150</v>
@@ -3467,10 +3560,10 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="C83" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="D83" t="s">
         <v>150</v>
@@ -3484,10 +3577,10 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C84" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="D84" t="s">
         <v>150</v>
@@ -3501,10 +3594,10 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C85" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="D85" t="s">
         <v>150</v>
@@ -3518,10 +3611,10 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="C86" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="D86" t="s">
         <v>150</v>
@@ -3535,10 +3628,10 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="C87" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="D87" t="s">
         <v>150</v>
@@ -3552,10 +3645,10 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C88" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="D88" t="s">
         <v>150</v>
@@ -3569,10 +3662,10 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="C89" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D89" t="s">
         <v>150</v>
@@ -3586,10 +3679,10 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C90" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="D90" t="s">
         <v>150</v>
@@ -3603,10 +3696,10 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="C91" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="D91" t="s">
         <v>150</v>
@@ -3620,10 +3713,10 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="C92" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="D92" t="s">
         <v>150</v>
@@ -3637,10 +3730,10 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C93" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D93" t="s">
         <v>150</v>
@@ -3654,10 +3747,10 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C94" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="D94" t="s">
         <v>150</v>
@@ -3671,10 +3764,10 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="C95" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D95" t="s">
         <v>150</v>
@@ -3688,10 +3781,10 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="C96" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="D96" t="s">
         <v>150</v>
@@ -3705,10 +3798,10 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="C97" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D97" t="s">
         <v>150</v>
@@ -3722,10 +3815,10 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="C98" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="D98" t="s">
         <v>150</v>
@@ -3739,10 +3832,10 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="C99" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D99" t="s">
         <v>150</v>
@@ -3756,10 +3849,10 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="C100" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="D100" t="s">
         <v>150</v>
@@ -3773,16 +3866,16 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C101" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="D101" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E101" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.3">
@@ -3790,16 +3883,16 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C102" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="D102" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E102" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.3">
@@ -3807,16 +3900,16 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="C103" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="D103" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E103" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.3">
@@ -3824,16 +3917,16 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="C104" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="D104" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E104" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.3">
@@ -3841,16 +3934,16 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>222</v>
+        <v>556</v>
       </c>
       <c r="C105" t="s">
-        <v>223</v>
+        <v>557</v>
       </c>
       <c r="D105" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E105" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.3">
@@ -3858,10 +3951,10 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="C106" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="D106" t="s">
         <v>215</v>
@@ -3875,10 +3968,10 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="C107" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="D107" t="s">
         <v>215</v>
@@ -3892,10 +3985,10 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="C108" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="D108" t="s">
         <v>215</v>
@@ -3909,10 +4002,10 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="C109" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="D109" t="s">
         <v>215</v>
@@ -3926,10 +4019,10 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="C110" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="D110" t="s">
         <v>215</v>
@@ -3943,10 +4036,10 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="C111" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="D111" t="s">
         <v>215</v>
@@ -3960,10 +4053,10 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="C112" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="D112" t="s">
         <v>215</v>
@@ -3977,10 +4070,10 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="C113" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="D113" t="s">
         <v>215</v>
@@ -3994,10 +4087,10 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C114" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="D114" t="s">
         <v>215</v>
@@ -4011,10 +4104,10 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="C115" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="D115" t="s">
         <v>215</v>
@@ -4028,10 +4121,10 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="C116" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="D116" t="s">
         <v>215</v>
@@ -4045,10 +4138,10 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="C117" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="D117" t="s">
         <v>215</v>
@@ -4062,10 +4155,10 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="C118" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="D118" t="s">
         <v>215</v>
@@ -4079,10 +4172,10 @@
         <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="C119" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="D119" t="s">
         <v>215</v>
@@ -4096,10 +4189,10 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="C120" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="D120" t="s">
         <v>215</v>
@@ -4113,10 +4206,10 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="C121" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="D121" t="s">
         <v>215</v>
@@ -4130,10 +4223,10 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="C122" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="D122" t="s">
         <v>215</v>
@@ -4147,10 +4240,10 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="C123" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="D123" t="s">
         <v>215</v>
@@ -4164,10 +4257,10 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="C124" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="D124" t="s">
         <v>215</v>
@@ -4181,10 +4274,10 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="C125" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="D125" t="s">
         <v>215</v>
@@ -4198,10 +4291,10 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="C126" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="D126" t="s">
         <v>215</v>
@@ -4215,10 +4308,10 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="C127" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="D127" t="s">
         <v>215</v>
@@ -4232,10 +4325,10 @@
         <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="C128" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="D128" t="s">
         <v>215</v>
@@ -4249,10 +4342,10 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="C129" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="D129" t="s">
         <v>215</v>
@@ -4266,10 +4359,10 @@
         <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="C130" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="D130" t="s">
         <v>215</v>
@@ -4283,10 +4376,10 @@
         <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="C131" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="D131" t="s">
         <v>215</v>
@@ -4300,10 +4393,10 @@
         <v>131</v>
       </c>
       <c r="B132" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="C132" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="D132" t="s">
         <v>215</v>
@@ -4317,16 +4410,16 @@
         <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="C133" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="D133" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E133" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.3">
@@ -4334,16 +4427,16 @@
         <v>133</v>
       </c>
       <c r="B134" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="C134" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="D134" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E134" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.3">
@@ -4351,16 +4444,16 @@
         <v>134</v>
       </c>
       <c r="B135" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="C135" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="D135" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E135" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.3">
@@ -4368,16 +4461,16 @@
         <v>135</v>
       </c>
       <c r="B136" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="C136" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="D136" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E136" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.3">
@@ -4385,16 +4478,16 @@
         <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="C137" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="D137" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E137" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.3">
@@ -4402,16 +4495,16 @@
         <v>137</v>
       </c>
       <c r="B138" t="s">
-        <v>288</v>
+        <v>558</v>
       </c>
       <c r="C138" t="s">
-        <v>289</v>
+        <v>559</v>
       </c>
       <c r="D138" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E138" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.3">
@@ -4419,16 +4512,16 @@
         <v>138</v>
       </c>
       <c r="B139" t="s">
-        <v>290</v>
+        <v>560</v>
       </c>
       <c r="C139" t="s">
-        <v>291</v>
+        <v>561</v>
       </c>
       <c r="D139" t="s">
         <v>4</v>
       </c>
       <c r="E139" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.3">
@@ -4436,10 +4529,10 @@
         <v>139</v>
       </c>
       <c r="B140" t="s">
-        <v>292</v>
+        <v>278</v>
       </c>
       <c r="C140" t="s">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="D140" t="s">
         <v>4</v>
@@ -4453,10 +4546,10 @@
         <v>140</v>
       </c>
       <c r="B141" t="s">
-        <v>294</v>
+        <v>280</v>
       </c>
       <c r="C141" t="s">
-        <v>295</v>
+        <v>281</v>
       </c>
       <c r="D141" t="s">
         <v>4</v>
@@ -4470,10 +4563,10 @@
         <v>141</v>
       </c>
       <c r="B142" t="s">
-        <v>296</v>
+        <v>282</v>
       </c>
       <c r="C142" t="s">
-        <v>297</v>
+        <v>283</v>
       </c>
       <c r="D142" t="s">
         <v>4</v>
@@ -4487,10 +4580,10 @@
         <v>142</v>
       </c>
       <c r="B143" t="s">
-        <v>298</v>
+        <v>284</v>
       </c>
       <c r="C143" t="s">
-        <v>299</v>
+        <v>285</v>
       </c>
       <c r="D143" t="s">
         <v>4</v>
@@ -4504,10 +4597,10 @@
         <v>143</v>
       </c>
       <c r="B144" t="s">
-        <v>300</v>
+        <v>286</v>
       </c>
       <c r="C144" t="s">
-        <v>301</v>
+        <v>287</v>
       </c>
       <c r="D144" t="s">
         <v>4</v>
@@ -4521,10 +4614,10 @@
         <v>144</v>
       </c>
       <c r="B145" t="s">
-        <v>302</v>
+        <v>288</v>
       </c>
       <c r="C145" t="s">
-        <v>303</v>
+        <v>289</v>
       </c>
       <c r="D145" t="s">
         <v>4</v>
@@ -4538,10 +4631,10 @@
         <v>145</v>
       </c>
       <c r="B146" t="s">
-        <v>304</v>
+        <v>290</v>
       </c>
       <c r="C146" t="s">
-        <v>305</v>
+        <v>291</v>
       </c>
       <c r="D146" t="s">
         <v>4</v>
@@ -4555,10 +4648,10 @@
         <v>146</v>
       </c>
       <c r="B147" t="s">
-        <v>306</v>
+        <v>292</v>
       </c>
       <c r="C147" t="s">
-        <v>307</v>
+        <v>293</v>
       </c>
       <c r="D147" t="s">
         <v>4</v>
@@ -4572,10 +4665,10 @@
         <v>147</v>
       </c>
       <c r="B148" t="s">
-        <v>308</v>
+        <v>294</v>
       </c>
       <c r="C148" t="s">
-        <v>309</v>
+        <v>295</v>
       </c>
       <c r="D148" t="s">
         <v>4</v>
@@ -4589,10 +4682,10 @@
         <v>148</v>
       </c>
       <c r="B149" t="s">
-        <v>310</v>
+        <v>296</v>
       </c>
       <c r="C149" t="s">
-        <v>311</v>
+        <v>297</v>
       </c>
       <c r="D149" t="s">
         <v>4</v>
@@ -4606,10 +4699,10 @@
         <v>149</v>
       </c>
       <c r="B150" t="s">
-        <v>312</v>
+        <v>298</v>
       </c>
       <c r="C150" t="s">
-        <v>313</v>
+        <v>299</v>
       </c>
       <c r="D150" t="s">
         <v>4</v>
@@ -4623,10 +4716,10 @@
         <v>150</v>
       </c>
       <c r="B151" t="s">
-        <v>314</v>
+        <v>300</v>
       </c>
       <c r="C151" t="s">
-        <v>315</v>
+        <v>301</v>
       </c>
       <c r="D151" t="s">
         <v>4</v>
@@ -4640,10 +4733,10 @@
         <v>151</v>
       </c>
       <c r="B152" t="s">
-        <v>316</v>
+        <v>302</v>
       </c>
       <c r="C152" t="s">
-        <v>317</v>
+        <v>303</v>
       </c>
       <c r="D152" t="s">
         <v>4</v>
@@ -4657,10 +4750,10 @@
         <v>152</v>
       </c>
       <c r="B153" t="s">
-        <v>318</v>
+        <v>304</v>
       </c>
       <c r="C153" t="s">
-        <v>319</v>
+        <v>305</v>
       </c>
       <c r="D153" t="s">
         <v>4</v>
@@ -4674,10 +4767,10 @@
         <v>153</v>
       </c>
       <c r="B154" t="s">
-        <v>320</v>
+        <v>306</v>
       </c>
       <c r="C154" t="s">
-        <v>321</v>
+        <v>307</v>
       </c>
       <c r="D154" t="s">
         <v>4</v>
@@ -4691,13 +4784,13 @@
         <v>154</v>
       </c>
       <c r="B155" t="s">
-        <v>322</v>
+        <v>308</v>
       </c>
       <c r="C155" t="s">
-        <v>323</v>
+        <v>309</v>
       </c>
       <c r="D155" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E155" t="s">
         <v>11</v>
@@ -4708,13 +4801,13 @@
         <v>155</v>
       </c>
       <c r="B156" t="s">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="C156" t="s">
-        <v>325</v>
+        <v>311</v>
       </c>
       <c r="D156" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E156" t="s">
         <v>11</v>
@@ -4725,13 +4818,13 @@
         <v>156</v>
       </c>
       <c r="B157" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="C157" t="s">
-        <v>327</v>
+        <v>313</v>
       </c>
       <c r="D157" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E157" t="s">
         <v>11</v>
@@ -4742,13 +4835,13 @@
         <v>157</v>
       </c>
       <c r="B158" t="s">
-        <v>328</v>
+        <v>314</v>
       </c>
       <c r="C158" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
       <c r="D158" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E158" t="s">
         <v>11</v>
@@ -4759,13 +4852,13 @@
         <v>158</v>
       </c>
       <c r="B159" t="s">
-        <v>330</v>
+        <v>316</v>
       </c>
       <c r="C159" t="s">
-        <v>331</v>
+        <v>317</v>
       </c>
       <c r="D159" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E159" t="s">
         <v>11</v>
@@ -4776,13 +4869,13 @@
         <v>159</v>
       </c>
       <c r="B160" t="s">
-        <v>332</v>
+        <v>318</v>
       </c>
       <c r="C160" t="s">
-        <v>333</v>
+        <v>319</v>
       </c>
       <c r="D160" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E160" t="s">
         <v>11</v>
@@ -4793,13 +4886,13 @@
         <v>160</v>
       </c>
       <c r="B161" t="s">
-        <v>334</v>
+        <v>320</v>
       </c>
       <c r="C161" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
       <c r="D161" t="s">
-        <v>215</v>
+        <v>4</v>
       </c>
       <c r="E161" t="s">
         <v>11</v>
@@ -4810,13 +4903,13 @@
         <v>161</v>
       </c>
       <c r="B162" t="s">
-        <v>336</v>
+        <v>322</v>
       </c>
       <c r="C162" t="s">
-        <v>337</v>
+        <v>323</v>
       </c>
       <c r="D162" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E162" t="s">
         <v>11</v>
@@ -4827,13 +4920,13 @@
         <v>162</v>
       </c>
       <c r="B163" t="s">
-        <v>338</v>
+        <v>324</v>
       </c>
       <c r="C163" t="s">
-        <v>339</v>
+        <v>325</v>
       </c>
       <c r="D163" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E163" t="s">
         <v>11</v>
@@ -4844,13 +4937,13 @@
         <v>163</v>
       </c>
       <c r="B164" t="s">
-        <v>340</v>
+        <v>326</v>
       </c>
       <c r="C164" t="s">
-        <v>341</v>
+        <v>327</v>
       </c>
       <c r="D164" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E164" t="s">
         <v>11</v>
@@ -4861,13 +4954,13 @@
         <v>164</v>
       </c>
       <c r="B165" t="s">
-        <v>342</v>
+        <v>328</v>
       </c>
       <c r="C165" t="s">
-        <v>343</v>
+        <v>329</v>
       </c>
       <c r="D165" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E165" t="s">
         <v>11</v>
@@ -4878,13 +4971,13 @@
         <v>165</v>
       </c>
       <c r="B166" t="s">
-        <v>344</v>
+        <v>330</v>
       </c>
       <c r="C166" t="s">
-        <v>345</v>
+        <v>331</v>
       </c>
       <c r="D166" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E166" t="s">
         <v>11</v>
@@ -4895,13 +4988,13 @@
         <v>166</v>
       </c>
       <c r="B167" t="s">
-        <v>346</v>
+        <v>332</v>
       </c>
       <c r="C167" t="s">
-        <v>347</v>
+        <v>333</v>
       </c>
       <c r="D167" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E167" t="s">
         <v>11</v>
@@ -4912,16 +5005,16 @@
         <v>167</v>
       </c>
       <c r="B168" t="s">
-        <v>348</v>
+        <v>334</v>
       </c>
       <c r="C168" t="s">
-        <v>349</v>
+        <v>335</v>
       </c>
       <c r="D168" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E168" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.3">
@@ -4929,16 +5022,16 @@
         <v>168</v>
       </c>
       <c r="B169" t="s">
-        <v>352</v>
+        <v>336</v>
       </c>
       <c r="C169" t="s">
-        <v>353</v>
+        <v>337</v>
       </c>
       <c r="D169" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E169" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.3">
@@ -4946,16 +5039,16 @@
         <v>169</v>
       </c>
       <c r="B170" t="s">
-        <v>354</v>
+        <v>338</v>
       </c>
       <c r="C170" t="s">
-        <v>355</v>
+        <v>339</v>
       </c>
       <c r="D170" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E170" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.3">
@@ -4963,16 +5056,16 @@
         <v>170</v>
       </c>
       <c r="B171" t="s">
-        <v>356</v>
+        <v>340</v>
       </c>
       <c r="C171" t="s">
-        <v>357</v>
+        <v>341</v>
       </c>
       <c r="D171" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E171" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.3">
@@ -4980,16 +5073,16 @@
         <v>171</v>
       </c>
       <c r="B172" t="s">
-        <v>358</v>
+        <v>342</v>
       </c>
       <c r="C172" t="s">
-        <v>359</v>
+        <v>343</v>
       </c>
       <c r="D172" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E172" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.3">
@@ -4997,16 +5090,16 @@
         <v>172</v>
       </c>
       <c r="B173" t="s">
-        <v>360</v>
+        <v>344</v>
       </c>
       <c r="C173" t="s">
-        <v>361</v>
+        <v>345</v>
       </c>
       <c r="D173" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E173" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.3">
@@ -5014,16 +5107,16 @@
         <v>173</v>
       </c>
       <c r="B174" t="s">
-        <v>362</v>
+        <v>346</v>
       </c>
       <c r="C174" t="s">
-        <v>363</v>
+        <v>347</v>
       </c>
       <c r="D174" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E174" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.3">
@@ -5031,10 +5124,10 @@
         <v>174</v>
       </c>
       <c r="B175" t="s">
-        <v>364</v>
+        <v>348</v>
       </c>
       <c r="C175" t="s">
-        <v>365</v>
+        <v>349</v>
       </c>
       <c r="D175" t="s">
         <v>350</v>
@@ -5048,10 +5141,10 @@
         <v>175</v>
       </c>
       <c r="B176" t="s">
-        <v>366</v>
+        <v>352</v>
       </c>
       <c r="C176" t="s">
-        <v>367</v>
+        <v>353</v>
       </c>
       <c r="D176" t="s">
         <v>350</v>
@@ -5065,10 +5158,10 @@
         <v>176</v>
       </c>
       <c r="B177" t="s">
-        <v>368</v>
+        <v>354</v>
       </c>
       <c r="C177" t="s">
-        <v>369</v>
+        <v>355</v>
       </c>
       <c r="D177" t="s">
         <v>350</v>
@@ -5082,10 +5175,10 @@
         <v>177</v>
       </c>
       <c r="B178" t="s">
-        <v>370</v>
+        <v>356</v>
       </c>
       <c r="C178" t="s">
-        <v>371</v>
+        <v>357</v>
       </c>
       <c r="D178" t="s">
         <v>350</v>
@@ -5099,10 +5192,10 @@
         <v>178</v>
       </c>
       <c r="B179" t="s">
-        <v>372</v>
+        <v>358</v>
       </c>
       <c r="C179" t="s">
-        <v>373</v>
+        <v>359</v>
       </c>
       <c r="D179" t="s">
         <v>350</v>
@@ -5116,10 +5209,10 @@
         <v>179</v>
       </c>
       <c r="B180" t="s">
-        <v>374</v>
+        <v>360</v>
       </c>
       <c r="C180" t="s">
-        <v>375</v>
+        <v>361</v>
       </c>
       <c r="D180" t="s">
         <v>350</v>
@@ -5133,10 +5226,10 @@
         <v>180</v>
       </c>
       <c r="B181" t="s">
-        <v>376</v>
+        <v>362</v>
       </c>
       <c r="C181" t="s">
-        <v>377</v>
+        <v>363</v>
       </c>
       <c r="D181" t="s">
         <v>350</v>
@@ -5150,10 +5243,10 @@
         <v>181</v>
       </c>
       <c r="B182" t="s">
-        <v>378</v>
+        <v>364</v>
       </c>
       <c r="C182" t="s">
-        <v>379</v>
+        <v>365</v>
       </c>
       <c r="D182" t="s">
         <v>350</v>
@@ -5167,10 +5260,10 @@
         <v>182</v>
       </c>
       <c r="B183" t="s">
-        <v>380</v>
+        <v>366</v>
       </c>
       <c r="C183" t="s">
-        <v>381</v>
+        <v>367</v>
       </c>
       <c r="D183" t="s">
         <v>350</v>
@@ -5184,10 +5277,10 @@
         <v>183</v>
       </c>
       <c r="B184" t="s">
-        <v>382</v>
+        <v>368</v>
       </c>
       <c r="C184" t="s">
-        <v>383</v>
+        <v>369</v>
       </c>
       <c r="D184" t="s">
         <v>350</v>
@@ -5201,10 +5294,10 @@
         <v>184</v>
       </c>
       <c r="B185" t="s">
-        <v>384</v>
+        <v>370</v>
       </c>
       <c r="C185" t="s">
-        <v>385</v>
+        <v>371</v>
       </c>
       <c r="D185" t="s">
         <v>350</v>
@@ -5218,10 +5311,10 @@
         <v>185</v>
       </c>
       <c r="B186" t="s">
-        <v>386</v>
+        <v>372</v>
       </c>
       <c r="C186" t="s">
-        <v>387</v>
+        <v>373</v>
       </c>
       <c r="D186" t="s">
         <v>350</v>
@@ -5235,10 +5328,10 @@
         <v>186</v>
       </c>
       <c r="B187" t="s">
-        <v>388</v>
+        <v>374</v>
       </c>
       <c r="C187" t="s">
-        <v>389</v>
+        <v>375</v>
       </c>
       <c r="D187" t="s">
         <v>350</v>
@@ -5252,10 +5345,10 @@
         <v>187</v>
       </c>
       <c r="B188" t="s">
-        <v>390</v>
+        <v>376</v>
       </c>
       <c r="C188" t="s">
-        <v>391</v>
+        <v>377</v>
       </c>
       <c r="D188" t="s">
         <v>350</v>
@@ -5269,10 +5362,10 @@
         <v>188</v>
       </c>
       <c r="B189" t="s">
-        <v>392</v>
+        <v>378</v>
       </c>
       <c r="C189" t="s">
-        <v>393</v>
+        <v>379</v>
       </c>
       <c r="D189" t="s">
         <v>350</v>
@@ -5286,10 +5379,10 @@
         <v>189</v>
       </c>
       <c r="B190" t="s">
-        <v>394</v>
+        <v>380</v>
       </c>
       <c r="C190" t="s">
-        <v>395</v>
+        <v>381</v>
       </c>
       <c r="D190" t="s">
         <v>350</v>
@@ -5303,10 +5396,10 @@
         <v>190</v>
       </c>
       <c r="B191" t="s">
-        <v>396</v>
+        <v>382</v>
       </c>
       <c r="C191" t="s">
-        <v>397</v>
+        <v>383</v>
       </c>
       <c r="D191" t="s">
         <v>350</v>
@@ -5320,10 +5413,10 @@
         <v>191</v>
       </c>
       <c r="B192" t="s">
-        <v>398</v>
+        <v>384</v>
       </c>
       <c r="C192" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="D192" t="s">
         <v>350</v>
@@ -5337,10 +5430,10 @@
         <v>192</v>
       </c>
       <c r="B193" t="s">
-        <v>400</v>
+        <v>386</v>
       </c>
       <c r="C193" t="s">
-        <v>401</v>
+        <v>387</v>
       </c>
       <c r="D193" t="s">
         <v>350</v>
@@ -5354,10 +5447,10 @@
         <v>193</v>
       </c>
       <c r="B194" t="s">
-        <v>402</v>
+        <v>388</v>
       </c>
       <c r="C194" t="s">
-        <v>403</v>
+        <v>389</v>
       </c>
       <c r="D194" t="s">
         <v>350</v>
@@ -5371,10 +5464,10 @@
         <v>194</v>
       </c>
       <c r="B195" t="s">
-        <v>404</v>
+        <v>390</v>
       </c>
       <c r="C195" t="s">
-        <v>405</v>
+        <v>391</v>
       </c>
       <c r="D195" t="s">
         <v>350</v>
@@ -5388,10 +5481,10 @@
         <v>195</v>
       </c>
       <c r="B196" t="s">
-        <v>406</v>
+        <v>392</v>
       </c>
       <c r="C196" t="s">
-        <v>407</v>
+        <v>393</v>
       </c>
       <c r="D196" t="s">
         <v>350</v>
@@ -5405,10 +5498,10 @@
         <v>196</v>
       </c>
       <c r="B197" t="s">
-        <v>408</v>
+        <v>394</v>
       </c>
       <c r="C197" t="s">
-        <v>409</v>
+        <v>395</v>
       </c>
       <c r="D197" t="s">
         <v>350</v>
@@ -5422,10 +5515,10 @@
         <v>197</v>
       </c>
       <c r="B198" t="s">
-        <v>410</v>
+        <v>396</v>
       </c>
       <c r="C198" t="s">
-        <v>411</v>
+        <v>397</v>
       </c>
       <c r="D198" t="s">
         <v>350</v>
@@ -5439,10 +5532,10 @@
         <v>198</v>
       </c>
       <c r="B199" t="s">
-        <v>412</v>
+        <v>398</v>
       </c>
       <c r="C199" t="s">
-        <v>413</v>
+        <v>399</v>
       </c>
       <c r="D199" t="s">
         <v>350</v>
@@ -5456,16 +5549,16 @@
         <v>199</v>
       </c>
       <c r="B200" t="s">
-        <v>414</v>
+        <v>400</v>
       </c>
       <c r="C200" t="s">
-        <v>415</v>
+        <v>401</v>
       </c>
       <c r="D200" t="s">
         <v>350</v>
       </c>
       <c r="E200" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.3">
@@ -5473,16 +5566,16 @@
         <v>200</v>
       </c>
       <c r="B201" t="s">
-        <v>417</v>
+        <v>402</v>
       </c>
       <c r="C201" t="s">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="D201" t="s">
         <v>350</v>
       </c>
       <c r="E201" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.3">
@@ -5490,16 +5583,16 @@
         <v>201</v>
       </c>
       <c r="B202" t="s">
-        <v>419</v>
+        <v>404</v>
       </c>
       <c r="C202" t="s">
-        <v>420</v>
+        <v>405</v>
       </c>
       <c r="D202" t="s">
         <v>350</v>
       </c>
       <c r="E202" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.3">
@@ -5507,16 +5600,16 @@
         <v>202</v>
       </c>
       <c r="B203" t="s">
-        <v>421</v>
+        <v>406</v>
       </c>
       <c r="C203" t="s">
-        <v>422</v>
+        <v>407</v>
       </c>
       <c r="D203" t="s">
         <v>350</v>
       </c>
       <c r="E203" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.3">
@@ -5524,16 +5617,16 @@
         <v>203</v>
       </c>
       <c r="B204" t="s">
-        <v>423</v>
+        <v>408</v>
       </c>
       <c r="C204" t="s">
-        <v>424</v>
+        <v>409</v>
       </c>
       <c r="D204" t="s">
         <v>350</v>
       </c>
       <c r="E204" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.3">
@@ -5541,16 +5634,16 @@
         <v>204</v>
       </c>
       <c r="B205" t="s">
-        <v>425</v>
+        <v>410</v>
       </c>
       <c r="C205" t="s">
-        <v>426</v>
+        <v>411</v>
       </c>
       <c r="D205" t="s">
         <v>350</v>
       </c>
       <c r="E205" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.3">
@@ -5558,16 +5651,16 @@
         <v>205</v>
       </c>
       <c r="B206" t="s">
-        <v>427</v>
+        <v>412</v>
       </c>
       <c r="C206" t="s">
-        <v>428</v>
+        <v>413</v>
       </c>
       <c r="D206" t="s">
         <v>350</v>
       </c>
       <c r="E206" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.3">
@@ -5575,10 +5668,10 @@
         <v>206</v>
       </c>
       <c r="B207" t="s">
-        <v>429</v>
+        <v>414</v>
       </c>
       <c r="C207" t="s">
-        <v>430</v>
+        <v>415</v>
       </c>
       <c r="D207" t="s">
         <v>350</v>
@@ -5592,10 +5685,10 @@
         <v>207</v>
       </c>
       <c r="B208" t="s">
-        <v>431</v>
+        <v>417</v>
       </c>
       <c r="C208" t="s">
-        <v>432</v>
+        <v>418</v>
       </c>
       <c r="D208" t="s">
         <v>350</v>
@@ -5609,10 +5702,10 @@
         <v>208</v>
       </c>
       <c r="B209" t="s">
-        <v>433</v>
+        <v>419</v>
       </c>
       <c r="C209" t="s">
-        <v>434</v>
+        <v>420</v>
       </c>
       <c r="D209" t="s">
         <v>350</v>
@@ -5626,10 +5719,10 @@
         <v>209</v>
       </c>
       <c r="B210" t="s">
-        <v>435</v>
+        <v>421</v>
       </c>
       <c r="C210" t="s">
-        <v>436</v>
+        <v>422</v>
       </c>
       <c r="D210" t="s">
         <v>350</v>
@@ -5643,10 +5736,10 @@
         <v>210</v>
       </c>
       <c r="B211" t="s">
-        <v>437</v>
+        <v>423</v>
       </c>
       <c r="C211" t="s">
-        <v>438</v>
+        <v>424</v>
       </c>
       <c r="D211" t="s">
         <v>350</v>
@@ -5660,10 +5753,10 @@
         <v>211</v>
       </c>
       <c r="B212" t="s">
-        <v>439</v>
+        <v>425</v>
       </c>
       <c r="C212" t="s">
-        <v>440</v>
+        <v>426</v>
       </c>
       <c r="D212" t="s">
         <v>350</v>
@@ -5677,13 +5770,13 @@
         <v>212</v>
       </c>
       <c r="B213" t="s">
-        <v>441</v>
+        <v>427</v>
       </c>
       <c r="C213" t="s">
-        <v>442</v>
+        <v>428</v>
       </c>
       <c r="D213" t="s">
-        <v>443</v>
+        <v>350</v>
       </c>
       <c r="E213" t="s">
         <v>416</v>
@@ -5694,13 +5787,13 @@
         <v>213</v>
       </c>
       <c r="B214" t="s">
-        <v>444</v>
+        <v>429</v>
       </c>
       <c r="C214" t="s">
-        <v>445</v>
+        <v>430</v>
       </c>
       <c r="D214" t="s">
-        <v>443</v>
+        <v>350</v>
       </c>
       <c r="E214" t="s">
         <v>416</v>
@@ -5711,13 +5804,13 @@
         <v>214</v>
       </c>
       <c r="B215" t="s">
-        <v>446</v>
+        <v>431</v>
       </c>
       <c r="C215" t="s">
-        <v>447</v>
+        <v>432</v>
       </c>
       <c r="D215" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E215" t="s">
         <v>416</v>
@@ -5728,13 +5821,13 @@
         <v>215</v>
       </c>
       <c r="B216" t="s">
-        <v>448</v>
+        <v>433</v>
       </c>
       <c r="C216" t="s">
-        <v>449</v>
+        <v>434</v>
       </c>
       <c r="D216" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E216" t="s">
         <v>416</v>
@@ -5745,13 +5838,13 @@
         <v>216</v>
       </c>
       <c r="B217" t="s">
-        <v>450</v>
+        <v>435</v>
       </c>
       <c r="C217" t="s">
-        <v>451</v>
+        <v>436</v>
       </c>
       <c r="D217" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E217" t="s">
         <v>416</v>
@@ -5762,13 +5855,13 @@
         <v>217</v>
       </c>
       <c r="B218" t="s">
-        <v>452</v>
+        <v>437</v>
       </c>
       <c r="C218" t="s">
-        <v>453</v>
+        <v>438</v>
       </c>
       <c r="D218" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E218" t="s">
         <v>416</v>
@@ -5779,13 +5872,13 @@
         <v>218</v>
       </c>
       <c r="B219" t="s">
-        <v>454</v>
+        <v>439</v>
       </c>
       <c r="C219" t="s">
-        <v>455</v>
+        <v>440</v>
       </c>
       <c r="D219" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E219" t="s">
         <v>416</v>
@@ -5796,13 +5889,13 @@
         <v>219</v>
       </c>
       <c r="B220" t="s">
-        <v>456</v>
+        <v>441</v>
       </c>
       <c r="C220" t="s">
-        <v>457</v>
+        <v>442</v>
       </c>
       <c r="D220" t="s">
-        <v>3</v>
+        <v>443</v>
       </c>
       <c r="E220" t="s">
         <v>416</v>
@@ -5813,13 +5906,13 @@
         <v>220</v>
       </c>
       <c r="B221" t="s">
-        <v>458</v>
+        <v>444</v>
       </c>
       <c r="C221" t="s">
-        <v>459</v>
+        <v>445</v>
       </c>
       <c r="D221" t="s">
-        <v>3</v>
+        <v>443</v>
       </c>
       <c r="E221" t="s">
         <v>416</v>
@@ -5830,10 +5923,10 @@
         <v>221</v>
       </c>
       <c r="B222" t="s">
-        <v>460</v>
+        <v>446</v>
       </c>
       <c r="C222" t="s">
-        <v>461</v>
+        <v>447</v>
       </c>
       <c r="D222" t="s">
         <v>3</v>
@@ -5847,10 +5940,10 @@
         <v>222</v>
       </c>
       <c r="B223" t="s">
-        <v>462</v>
+        <v>448</v>
       </c>
       <c r="C223" t="s">
-        <v>463</v>
+        <v>449</v>
       </c>
       <c r="D223" t="s">
         <v>3</v>
@@ -5864,10 +5957,10 @@
         <v>223</v>
       </c>
       <c r="B224" t="s">
-        <v>464</v>
+        <v>450</v>
       </c>
       <c r="C224" t="s">
-        <v>465</v>
+        <v>451</v>
       </c>
       <c r="D224" t="s">
         <v>3</v>
@@ -5881,13 +5974,13 @@
         <v>224</v>
       </c>
       <c r="B225" t="s">
-        <v>466</v>
+        <v>452</v>
       </c>
       <c r="C225" t="s">
-        <v>467</v>
+        <v>453</v>
       </c>
       <c r="D225" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E225" t="s">
         <v>416</v>
@@ -5898,13 +5991,13 @@
         <v>225</v>
       </c>
       <c r="B226" t="s">
-        <v>469</v>
+        <v>454</v>
       </c>
       <c r="C226" t="s">
-        <v>470</v>
+        <v>455</v>
       </c>
       <c r="D226" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E226" t="s">
         <v>416</v>
@@ -5915,13 +6008,13 @@
         <v>226</v>
       </c>
       <c r="B227" t="s">
-        <v>471</v>
+        <v>456</v>
       </c>
       <c r="C227" t="s">
-        <v>472</v>
+        <v>457</v>
       </c>
       <c r="D227" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E227" t="s">
         <v>416</v>
@@ -5932,13 +6025,13 @@
         <v>227</v>
       </c>
       <c r="B228" t="s">
-        <v>473</v>
+        <v>458</v>
       </c>
       <c r="C228" t="s">
-        <v>474</v>
+        <v>459</v>
       </c>
       <c r="D228" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E228" t="s">
         <v>416</v>
@@ -5949,13 +6042,13 @@
         <v>228</v>
       </c>
       <c r="B229" t="s">
-        <v>475</v>
+        <v>460</v>
       </c>
       <c r="C229" t="s">
-        <v>476</v>
+        <v>461</v>
       </c>
       <c r="D229" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E229" t="s">
         <v>416</v>
@@ -5966,13 +6059,13 @@
         <v>229</v>
       </c>
       <c r="B230" t="s">
-        <v>477</v>
+        <v>462</v>
       </c>
       <c r="C230" t="s">
-        <v>478</v>
+        <v>463</v>
       </c>
       <c r="D230" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E230" t="s">
         <v>416</v>
@@ -5983,13 +6076,13 @@
         <v>230</v>
       </c>
       <c r="B231" t="s">
-        <v>479</v>
+        <v>464</v>
       </c>
       <c r="C231" t="s">
-        <v>480</v>
+        <v>465</v>
       </c>
       <c r="D231" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E231" t="s">
         <v>416</v>
@@ -6000,13 +6093,13 @@
         <v>231</v>
       </c>
       <c r="B232" t="s">
-        <v>481</v>
+        <v>562</v>
       </c>
       <c r="C232" t="s">
-        <v>482</v>
+        <v>563</v>
       </c>
       <c r="D232" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E232" t="s">
         <v>416</v>
@@ -6017,10 +6110,10 @@
         <v>232</v>
       </c>
       <c r="B233" t="s">
-        <v>483</v>
+        <v>466</v>
       </c>
       <c r="C233" t="s">
-        <v>484</v>
+        <v>467</v>
       </c>
       <c r="D233" t="s">
         <v>468</v>
@@ -6034,16 +6127,16 @@
         <v>233</v>
       </c>
       <c r="B234" t="s">
-        <v>485</v>
+        <v>469</v>
       </c>
       <c r="C234" t="s">
-        <v>486</v>
+        <v>470</v>
       </c>
       <c r="D234" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E234" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.3">
@@ -6051,16 +6144,16 @@
         <v>234</v>
       </c>
       <c r="B235" t="s">
-        <v>489</v>
+        <v>471</v>
       </c>
       <c r="C235" t="s">
-        <v>490</v>
+        <v>472</v>
       </c>
       <c r="D235" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E235" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="236" spans="1:5" x14ac:dyDescent="0.3">
@@ -6068,16 +6161,16 @@
         <v>235</v>
       </c>
       <c r="B236" t="s">
-        <v>491</v>
+        <v>473</v>
       </c>
       <c r="C236" t="s">
-        <v>492</v>
+        <v>474</v>
       </c>
       <c r="D236" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E236" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="237" spans="1:5" x14ac:dyDescent="0.3">
@@ -6085,16 +6178,16 @@
         <v>236</v>
       </c>
       <c r="B237" t="s">
-        <v>493</v>
+        <v>475</v>
       </c>
       <c r="C237" t="s">
-        <v>494</v>
+        <v>476</v>
       </c>
       <c r="D237" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E237" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="238" spans="1:5" x14ac:dyDescent="0.3">
@@ -6102,16 +6195,16 @@
         <v>237</v>
       </c>
       <c r="B238" t="s">
-        <v>495</v>
+        <v>477</v>
       </c>
       <c r="C238" t="s">
-        <v>496</v>
+        <v>478</v>
       </c>
       <c r="D238" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E238" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="239" spans="1:5" x14ac:dyDescent="0.3">
@@ -6119,16 +6212,16 @@
         <v>238</v>
       </c>
       <c r="B239" t="s">
-        <v>497</v>
+        <v>479</v>
       </c>
       <c r="C239" t="s">
-        <v>498</v>
+        <v>480</v>
       </c>
       <c r="D239" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E239" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="240" spans="1:5" x14ac:dyDescent="0.3">
@@ -6136,16 +6229,16 @@
         <v>239</v>
       </c>
       <c r="B240" t="s">
-        <v>499</v>
+        <v>481</v>
       </c>
       <c r="C240" t="s">
-        <v>500</v>
+        <v>482</v>
       </c>
       <c r="D240" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E240" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="241" spans="1:5" x14ac:dyDescent="0.3">
@@ -6153,16 +6246,16 @@
         <v>240</v>
       </c>
       <c r="B241" t="s">
-        <v>501</v>
+        <v>483</v>
       </c>
       <c r="C241" t="s">
-        <v>502</v>
+        <v>484</v>
       </c>
       <c r="D241" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E241" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="242" spans="1:5" x14ac:dyDescent="0.3">
@@ -6170,10 +6263,10 @@
         <v>241</v>
       </c>
       <c r="B242" t="s">
-        <v>503</v>
+        <v>485</v>
       </c>
       <c r="C242" t="s">
-        <v>504</v>
+        <v>486</v>
       </c>
       <c r="D242" t="s">
         <v>487</v>
@@ -6187,10 +6280,10 @@
         <v>242</v>
       </c>
       <c r="B243" t="s">
-        <v>505</v>
+        <v>489</v>
       </c>
       <c r="C243" t="s">
-        <v>506</v>
+        <v>490</v>
       </c>
       <c r="D243" t="s">
         <v>487</v>
@@ -6204,13 +6297,13 @@
         <v>243</v>
       </c>
       <c r="B244" t="s">
-        <v>507</v>
+        <v>491</v>
       </c>
       <c r="C244" t="s">
-        <v>508</v>
+        <v>492</v>
       </c>
       <c r="D244" t="s">
-        <v>509</v>
+        <v>487</v>
       </c>
       <c r="E244" t="s">
         <v>488</v>
@@ -6221,13 +6314,13 @@
         <v>244</v>
       </c>
       <c r="B245" t="s">
-        <v>510</v>
+        <v>493</v>
       </c>
       <c r="C245" t="s">
-        <v>511</v>
+        <v>494</v>
       </c>
       <c r="D245" t="s">
-        <v>509</v>
+        <v>487</v>
       </c>
       <c r="E245" t="s">
         <v>488</v>
@@ -6238,13 +6331,13 @@
         <v>245</v>
       </c>
       <c r="B246" t="s">
-        <v>512</v>
+        <v>495</v>
       </c>
       <c r="C246" t="s">
-        <v>513</v>
+        <v>496</v>
       </c>
       <c r="D246" t="s">
-        <v>514</v>
+        <v>487</v>
       </c>
       <c r="E246" t="s">
         <v>488</v>
@@ -6255,13 +6348,13 @@
         <v>246</v>
       </c>
       <c r="B247" t="s">
-        <v>515</v>
+        <v>497</v>
       </c>
       <c r="C247" t="s">
-        <v>516</v>
+        <v>498</v>
       </c>
       <c r="D247" t="s">
-        <v>514</v>
+        <v>487</v>
       </c>
       <c r="E247" t="s">
         <v>488</v>
@@ -6272,13 +6365,13 @@
         <v>247</v>
       </c>
       <c r="B248" t="s">
-        <v>517</v>
+        <v>499</v>
       </c>
       <c r="C248" t="s">
-        <v>518</v>
+        <v>500</v>
       </c>
       <c r="D248" t="s">
-        <v>514</v>
+        <v>487</v>
       </c>
       <c r="E248" t="s">
         <v>488</v>
@@ -6289,13 +6382,13 @@
         <v>248</v>
       </c>
       <c r="B249" t="s">
-        <v>519</v>
+        <v>501</v>
       </c>
       <c r="C249" t="s">
-        <v>520</v>
+        <v>502</v>
       </c>
       <c r="D249" t="s">
-        <v>521</v>
+        <v>487</v>
       </c>
       <c r="E249" t="s">
         <v>488</v>
@@ -6306,13 +6399,13 @@
         <v>249</v>
       </c>
       <c r="B250" t="s">
-        <v>522</v>
+        <v>503</v>
       </c>
       <c r="C250" t="s">
-        <v>523</v>
+        <v>504</v>
       </c>
       <c r="D250" t="s">
-        <v>521</v>
+        <v>487</v>
       </c>
       <c r="E250" t="s">
         <v>488</v>
@@ -6323,13 +6416,13 @@
         <v>250</v>
       </c>
       <c r="B251" t="s">
-        <v>524</v>
+        <v>505</v>
       </c>
       <c r="C251" t="s">
-        <v>525</v>
+        <v>506</v>
       </c>
       <c r="D251" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="E251" t="s">
         <v>488</v>
@@ -6340,13 +6433,13 @@
         <v>251</v>
       </c>
       <c r="B252" t="s">
-        <v>527</v>
+        <v>564</v>
       </c>
       <c r="C252" t="s">
-        <v>528</v>
+        <v>565</v>
       </c>
       <c r="D252" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="E252" t="s">
         <v>488</v>
@@ -6357,13 +6450,13 @@
         <v>252</v>
       </c>
       <c r="B253" t="s">
-        <v>529</v>
+        <v>566</v>
       </c>
       <c r="C253" t="s">
-        <v>530</v>
+        <v>567</v>
       </c>
       <c r="D253" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="E253" t="s">
         <v>488</v>
@@ -6374,13 +6467,13 @@
         <v>253</v>
       </c>
       <c r="B254" t="s">
-        <v>531</v>
+        <v>507</v>
       </c>
       <c r="C254" t="s">
-        <v>532</v>
+        <v>508</v>
       </c>
       <c r="D254" t="s">
-        <v>526</v>
+        <v>509</v>
       </c>
       <c r="E254" t="s">
         <v>488</v>
@@ -6391,13 +6484,13 @@
         <v>254</v>
       </c>
       <c r="B255" t="s">
-        <v>533</v>
+        <v>510</v>
       </c>
       <c r="C255" t="s">
-        <v>534</v>
+        <v>511</v>
       </c>
       <c r="D255" t="s">
-        <v>526</v>
+        <v>509</v>
       </c>
       <c r="E255" t="s">
         <v>488</v>
@@ -6408,13 +6501,13 @@
         <v>255</v>
       </c>
       <c r="B256" t="s">
-        <v>535</v>
+        <v>512</v>
       </c>
       <c r="C256" t="s">
-        <v>536</v>
+        <v>513</v>
       </c>
       <c r="D256" t="s">
-        <v>526</v>
+        <v>514</v>
       </c>
       <c r="E256" t="s">
         <v>488</v>
@@ -6425,13 +6518,13 @@
         <v>256</v>
       </c>
       <c r="B257" t="s">
-        <v>537</v>
+        <v>515</v>
       </c>
       <c r="C257" t="s">
-        <v>538</v>
+        <v>516</v>
       </c>
       <c r="D257" t="s">
-        <v>526</v>
+        <v>514</v>
       </c>
       <c r="E257" t="s">
         <v>488</v>
@@ -6442,13 +6535,13 @@
         <v>257</v>
       </c>
       <c r="B258" t="s">
-        <v>539</v>
+        <v>517</v>
       </c>
       <c r="C258" t="s">
-        <v>540</v>
+        <v>518</v>
       </c>
       <c r="D258" t="s">
-        <v>526</v>
+        <v>514</v>
       </c>
       <c r="E258" t="s">
         <v>488</v>
@@ -6459,13 +6552,13 @@
         <v>258</v>
       </c>
       <c r="B259" t="s">
-        <v>541</v>
+        <v>519</v>
       </c>
       <c r="C259" t="s">
-        <v>542</v>
+        <v>520</v>
       </c>
       <c r="D259" t="s">
-        <v>543</v>
+        <v>521</v>
       </c>
       <c r="E259" t="s">
         <v>488</v>
@@ -6476,13 +6569,13 @@
         <v>259</v>
       </c>
       <c r="B260" t="s">
-        <v>544</v>
+        <v>522</v>
       </c>
       <c r="C260" t="s">
-        <v>545</v>
+        <v>523</v>
       </c>
       <c r="D260" t="s">
-        <v>543</v>
+        <v>521</v>
       </c>
       <c r="E260" t="s">
         <v>488</v>
@@ -6493,15 +6586,270 @@
         <v>260</v>
       </c>
       <c r="B261" t="s">
+        <v>568</v>
+      </c>
+      <c r="C261" t="s">
+        <v>569</v>
+      </c>
+      <c r="D261" t="s">
+        <v>521</v>
+      </c>
+      <c r="E261" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="262" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A262">
+        <v>261</v>
+      </c>
+      <c r="B262" t="s">
+        <v>570</v>
+      </c>
+      <c r="C262" t="s">
+        <v>571</v>
+      </c>
+      <c r="D262" t="s">
+        <v>521</v>
+      </c>
+      <c r="E262" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="263" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A263">
+        <v>262</v>
+      </c>
+      <c r="B263" t="s">
+        <v>524</v>
+      </c>
+      <c r="C263" t="s">
+        <v>525</v>
+      </c>
+      <c r="D263" t="s">
+        <v>526</v>
+      </c>
+      <c r="E263" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="264" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A264">
+        <v>263</v>
+      </c>
+      <c r="B264" t="s">
+        <v>527</v>
+      </c>
+      <c r="C264" t="s">
+        <v>528</v>
+      </c>
+      <c r="D264" t="s">
+        <v>526</v>
+      </c>
+      <c r="E264" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="265" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A265">
+        <v>264</v>
+      </c>
+      <c r="B265" t="s">
+        <v>529</v>
+      </c>
+      <c r="C265" t="s">
+        <v>530</v>
+      </c>
+      <c r="D265" t="s">
+        <v>526</v>
+      </c>
+      <c r="E265" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="266" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A266">
+        <v>265</v>
+      </c>
+      <c r="B266" t="s">
+        <v>531</v>
+      </c>
+      <c r="C266" t="s">
+        <v>532</v>
+      </c>
+      <c r="D266" t="s">
+        <v>526</v>
+      </c>
+      <c r="E266" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="267" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A267">
+        <v>266</v>
+      </c>
+      <c r="B267" t="s">
+        <v>533</v>
+      </c>
+      <c r="C267" t="s">
+        <v>534</v>
+      </c>
+      <c r="D267" t="s">
+        <v>526</v>
+      </c>
+      <c r="E267" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="268" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A268">
+        <v>267</v>
+      </c>
+      <c r="B268" t="s">
+        <v>535</v>
+      </c>
+      <c r="C268" t="s">
+        <v>536</v>
+      </c>
+      <c r="D268" t="s">
+        <v>526</v>
+      </c>
+      <c r="E268" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="269" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A269">
+        <v>268</v>
+      </c>
+      <c r="B269" t="s">
+        <v>537</v>
+      </c>
+      <c r="C269" t="s">
+        <v>538</v>
+      </c>
+      <c r="D269" t="s">
+        <v>526</v>
+      </c>
+      <c r="E269" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="270" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A270">
+        <v>269</v>
+      </c>
+      <c r="B270" t="s">
+        <v>539</v>
+      </c>
+      <c r="C270" t="s">
+        <v>540</v>
+      </c>
+      <c r="D270" t="s">
+        <v>526</v>
+      </c>
+      <c r="E270" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="271" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A271">
+        <v>270</v>
+      </c>
+      <c r="B271" t="s">
+        <v>541</v>
+      </c>
+      <c r="C271" t="s">
+        <v>542</v>
+      </c>
+      <c r="D271" t="s">
+        <v>543</v>
+      </c>
+      <c r="E271" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="272" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A272">
+        <v>271</v>
+      </c>
+      <c r="B272" t="s">
+        <v>544</v>
+      </c>
+      <c r="C272" t="s">
+        <v>545</v>
+      </c>
+      <c r="D272" t="s">
+        <v>543</v>
+      </c>
+      <c r="E272" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="273" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A273">
+        <v>272</v>
+      </c>
+      <c r="B273" t="s">
         <v>546</v>
       </c>
-      <c r="C261" t="s">
+      <c r="C273" t="s">
         <v>547</v>
       </c>
-      <c r="D261" t="s">
+      <c r="D273" t="s">
         <v>543</v>
       </c>
-      <c r="E261" t="s">
+      <c r="E273" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="274" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A274">
+        <v>273</v>
+      </c>
+      <c r="B274" t="s">
+        <v>572</v>
+      </c>
+      <c r="C274" t="s">
+        <v>573</v>
+      </c>
+      <c r="D274" t="s">
+        <v>350</v>
+      </c>
+      <c r="E274" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="275" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A275">
+        <v>274</v>
+      </c>
+      <c r="B275" t="s">
+        <v>574</v>
+      </c>
+      <c r="C275" t="s">
+        <v>575</v>
+      </c>
+      <c r="D275" t="s">
+        <v>468</v>
+      </c>
+      <c r="E275" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="276" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A276">
+        <v>275</v>
+      </c>
+      <c r="B276" t="s">
+        <v>576</v>
+      </c>
+      <c r="C276" t="s">
+        <v>577</v>
+      </c>
+      <c r="D276" t="s">
+        <v>578</v>
+      </c>
+      <c r="E276" t="s">
         <v>488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update roster to 301 students
Regenerate data.js from the latest Students Details.xlsx. Note:
generate_data.py's duplicate-PRN check flagged SEFU126011 used by two
different students (see WARNING at generation time) — needs a fix in
the source spreadsheet, not something this script can resolve.
</commit_message>
<xml_diff>
--- a/Students Details.xlsx
+++ b/Students Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Krishnendu.Jana\Desktop\MITVPU-Orientation-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E534BB-9B99-4F64-A8DB-EC9227FAD183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F18D39F3-CE26-4DC5-A83D-B317BCE8B4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7991DB97-C80E-432A-B6FF-7E61A06C8A94}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="630">
   <si>
     <t>PRN</t>
   </si>
@@ -1776,6 +1776,159 @@
   </si>
   <si>
     <t>B. Pharm. LE</t>
+  </si>
+  <si>
+    <t>SCFP126059</t>
+  </si>
+  <si>
+    <t>Koli Sapana Mahadev</t>
+  </si>
+  <si>
+    <t>SCFP126060</t>
+  </si>
+  <si>
+    <t>Gaddam Akash Chandrakant</t>
+  </si>
+  <si>
+    <t>SCFU426025</t>
+  </si>
+  <si>
+    <t>Singham Onkar Jalindar</t>
+  </si>
+  <si>
+    <t>SCFU426026</t>
+  </si>
+  <si>
+    <t>Relekar Dhanashri Siddharth</t>
+  </si>
+  <si>
+    <t>SCFU126040</t>
+  </si>
+  <si>
+    <t>Rathod Om Raosaheb</t>
+  </si>
+  <si>
+    <t>SCFU126041</t>
+  </si>
+  <si>
+    <t>Gangavkar Nikhilesh Prashant</t>
+  </si>
+  <si>
+    <t>SCFU126042</t>
+  </si>
+  <si>
+    <t>Adone Utkarsha Gopal</t>
+  </si>
+  <si>
+    <t>SCFU126043</t>
+  </si>
+  <si>
+    <t>Nikhi Kumar</t>
+  </si>
+  <si>
+    <t>SCFU126044</t>
+  </si>
+  <si>
+    <t>Aman Irshad husain Zartar</t>
+  </si>
+  <si>
+    <t>SCFU126045</t>
+  </si>
+  <si>
+    <t>Abdul Zaid</t>
+  </si>
+  <si>
+    <t>SCLU326041</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Shraddha Chandrashekhar Minajagi</t>
+  </si>
+  <si>
+    <t>SCLU326042</t>
+  </si>
+  <si>
+    <t>Kota Akshara Gyaneshwar</t>
+  </si>
+  <si>
+    <t>SCLU326043</t>
+  </si>
+  <si>
+    <t>Badepeer Rayyan Shakil</t>
+  </si>
+  <si>
+    <t>SCLU326044</t>
+  </si>
+  <si>
+    <t>Bhimpure Pramod Prashnat</t>
+  </si>
+  <si>
+    <t>SCLU326045</t>
+  </si>
+  <si>
+    <t>Kshirsagar Sumedh Avinash</t>
+  </si>
+  <si>
+    <t>SCFU226012</t>
+  </si>
+  <si>
+    <t>Swami Spoorti Amitkumar</t>
+  </si>
+  <si>
+    <t>SELU126005</t>
+  </si>
+  <si>
+    <t>Battul Shrutika Nardendra</t>
+  </si>
+  <si>
+    <t>Nade Ashutosh Abhijit</t>
+  </si>
+  <si>
+    <t>BSFP126011</t>
+  </si>
+  <si>
+    <t>Jadhav Sonali Sukhdev</t>
+  </si>
+  <si>
+    <t>SPFU126004</t>
+  </si>
+  <si>
+    <t>Singh Yogita</t>
+  </si>
+  <si>
+    <t>BSFP226013</t>
+  </si>
+  <si>
+    <t>Fulari Nagendra Kashinath</t>
+  </si>
+  <si>
+    <t>BSFP226014</t>
+  </si>
+  <si>
+    <t>Rampure Onkar Ramesh</t>
+  </si>
+  <si>
+    <t>BSFU126047</t>
+  </si>
+  <si>
+    <t>Vaychal Santosh Sarthak</t>
+  </si>
+  <si>
+    <t>BSFU126048</t>
+  </si>
+  <si>
+    <t>Charudatta Ajay Naik</t>
+  </si>
+  <si>
+    <t>BSFU126049</t>
+  </si>
+  <si>
+    <t>Holagi Gangadhar Shantappa</t>
+  </si>
+  <si>
+    <t>BSFU126050</t>
+  </si>
+  <si>
+    <t>Kshirsagar Aryan Amar</t>
   </si>
 </sst>
 </file>
@@ -2153,7 +2306,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81D7E270-40BB-453E-AA25-D300316939A2}">
-  <dimension ref="A1:E276"/>
+  <dimension ref="A1:E302"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
@@ -2778,16 +2931,16 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>82</v>
+        <v>579</v>
       </c>
       <c r="C37" t="s">
-        <v>83</v>
+        <v>580</v>
       </c>
       <c r="D37" t="s">
-        <v>84</v>
+        <v>4</v>
       </c>
       <c r="E37" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
@@ -2795,16 +2948,16 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>85</v>
+        <v>581</v>
       </c>
       <c r="C38" t="s">
-        <v>86</v>
+        <v>582</v>
       </c>
       <c r="D38" t="s">
-        <v>84</v>
+        <v>4</v>
       </c>
       <c r="E38" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
@@ -2812,16 +2965,16 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>87</v>
+        <v>583</v>
       </c>
       <c r="C39" t="s">
-        <v>88</v>
+        <v>584</v>
       </c>
       <c r="D39" t="s">
         <v>84</v>
       </c>
       <c r="E39" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
@@ -2829,16 +2982,16 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>89</v>
+        <v>585</v>
       </c>
       <c r="C40" t="s">
-        <v>90</v>
+        <v>586</v>
       </c>
       <c r="D40" t="s">
         <v>84</v>
       </c>
       <c r="E40" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
@@ -2846,10 +2999,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="C41" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="D41" t="s">
         <v>84</v>
@@ -2863,10 +3016,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="C42" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="D42" t="s">
         <v>84</v>
@@ -2880,10 +3033,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C43" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="D43" t="s">
         <v>84</v>
@@ -2897,10 +3050,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C44" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="D44" t="s">
         <v>84</v>
@@ -2914,10 +3067,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C45" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="D45" t="s">
         <v>84</v>
@@ -2931,10 +3084,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C46" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="D46" t="s">
         <v>84</v>
@@ -2948,10 +3101,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="C47" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D47" t="s">
         <v>84</v>
@@ -2965,10 +3118,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="C48" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D48" t="s">
         <v>84</v>
@@ -2982,10 +3135,10 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C49" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D49" t="s">
         <v>84</v>
@@ -2999,10 +3152,10 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="C50" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D50" t="s">
         <v>84</v>
@@ -3016,10 +3169,10 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="C51" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="D51" t="s">
         <v>84</v>
@@ -3033,10 +3186,10 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C52" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="D52" t="s">
         <v>84</v>
@@ -3050,10 +3203,10 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C53" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="D53" t="s">
         <v>84</v>
@@ -3067,10 +3220,10 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C54" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="D54" t="s">
         <v>84</v>
@@ -3084,10 +3237,10 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C55" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="D55" t="s">
         <v>84</v>
@@ -3101,10 +3254,10 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="C56" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="D56" t="s">
         <v>84</v>
@@ -3118,10 +3271,10 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C57" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D57" t="s">
         <v>84</v>
@@ -3135,10 +3288,10 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C58" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D58" t="s">
         <v>84</v>
@@ -3152,10 +3305,10 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="C59" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="D59" t="s">
         <v>84</v>
@@ -3169,10 +3322,10 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>548</v>
+        <v>121</v>
       </c>
       <c r="C60" t="s">
-        <v>549</v>
+        <v>122</v>
       </c>
       <c r="D60" t="s">
         <v>84</v>
@@ -3186,13 +3339,13 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="C61" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="D61" t="s">
-        <v>131</v>
+        <v>84</v>
       </c>
       <c r="E61" t="s">
         <v>8</v>
@@ -3203,13 +3356,13 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="C62" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="D62" t="s">
-        <v>131</v>
+        <v>84</v>
       </c>
       <c r="E62" t="s">
         <v>8</v>
@@ -3220,13 +3373,13 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="C63" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D63" t="s">
-        <v>131</v>
+        <v>84</v>
       </c>
       <c r="E63" t="s">
         <v>8</v>
@@ -3237,13 +3390,13 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>136</v>
+        <v>548</v>
       </c>
       <c r="C64" t="s">
-        <v>137</v>
+        <v>549</v>
       </c>
       <c r="D64" t="s">
-        <v>131</v>
+        <v>84</v>
       </c>
       <c r="E64" t="s">
         <v>8</v>
@@ -3254,10 +3407,10 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="C65" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="D65" t="s">
         <v>131</v>
@@ -3271,10 +3424,10 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="C66" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="D66" t="s">
         <v>131</v>
@@ -3288,10 +3441,10 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="C67" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="D67" t="s">
         <v>131</v>
@@ -3305,10 +3458,10 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="C68" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="D68" t="s">
         <v>131</v>
@@ -3322,10 +3475,10 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C69" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="D69" t="s">
         <v>131</v>
@@ -3339,10 +3492,10 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>550</v>
+        <v>140</v>
       </c>
       <c r="C70" t="s">
-        <v>551</v>
+        <v>141</v>
       </c>
       <c r="D70" t="s">
         <v>131</v>
@@ -3356,10 +3509,10 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>552</v>
+        <v>142</v>
       </c>
       <c r="C71" t="s">
-        <v>553</v>
+        <v>143</v>
       </c>
       <c r="D71" t="s">
         <v>131</v>
@@ -3373,10 +3526,10 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>554</v>
+        <v>144</v>
       </c>
       <c r="C72" t="s">
-        <v>555</v>
+        <v>145</v>
       </c>
       <c r="D72" t="s">
         <v>131</v>
@@ -3390,16 +3543,16 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C73" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D73" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="E73" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
@@ -3407,16 +3560,16 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>151</v>
+        <v>550</v>
       </c>
       <c r="C74" t="s">
-        <v>152</v>
+        <v>551</v>
       </c>
       <c r="D74" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="E74" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
@@ -3424,16 +3577,16 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>153</v>
+        <v>552</v>
       </c>
       <c r="C75" t="s">
-        <v>154</v>
+        <v>553</v>
       </c>
       <c r="D75" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="E75" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
@@ -3441,16 +3594,16 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>155</v>
+        <v>554</v>
       </c>
       <c r="C76" t="s">
-        <v>156</v>
+        <v>555</v>
       </c>
       <c r="D76" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="E76" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
@@ -3458,10 +3611,10 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="C77" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
       <c r="D77" t="s">
         <v>150</v>
@@ -3475,10 +3628,10 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C78" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="D78" t="s">
         <v>150</v>
@@ -3492,10 +3645,10 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="C79" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D79" t="s">
         <v>150</v>
@@ -3509,10 +3662,10 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="C80" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="D80" t="s">
         <v>150</v>
@@ -3526,10 +3679,10 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="C81" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="D81" t="s">
         <v>150</v>
@@ -3543,10 +3696,10 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C82" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D82" t="s">
         <v>150</v>
@@ -3560,10 +3713,10 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="C83" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="D83" t="s">
         <v>150</v>
@@ -3577,10 +3730,10 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="C84" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D84" t="s">
         <v>150</v>
@@ -3594,10 +3747,10 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="C85" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="D85" t="s">
         <v>150</v>
@@ -3611,10 +3764,10 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="C86" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="D86" t="s">
         <v>150</v>
@@ -3628,10 +3781,10 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="C87" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="D87" t="s">
         <v>150</v>
@@ -3645,10 +3798,10 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C88" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="D88" t="s">
         <v>150</v>
@@ -3662,10 +3815,10 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C89" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="D89" t="s">
         <v>150</v>
@@ -3679,10 +3832,10 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="C90" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="D90" t="s">
         <v>150</v>
@@ -3696,10 +3849,10 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="C91" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="D91" t="s">
         <v>150</v>
@@ -3713,10 +3866,10 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C92" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="D92" t="s">
         <v>150</v>
@@ -3730,10 +3883,10 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="C93" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D93" t="s">
         <v>150</v>
@@ -3747,10 +3900,10 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C94" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="D94" t="s">
         <v>150</v>
@@ -3764,10 +3917,10 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="C95" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="D95" t="s">
         <v>150</v>
@@ -3781,10 +3934,10 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="C96" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="D96" t="s">
         <v>150</v>
@@ -3798,10 +3951,10 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C97" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="D97" t="s">
         <v>150</v>
@@ -3815,10 +3968,10 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C98" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="D98" t="s">
         <v>150</v>
@@ -3832,10 +3985,10 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="C99" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D99" t="s">
         <v>150</v>
@@ -3849,10 +4002,10 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="C100" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="D100" t="s">
         <v>150</v>
@@ -3866,10 +4019,10 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="C101" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D101" t="s">
         <v>150</v>
@@ -3883,10 +4036,10 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="C102" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="D102" t="s">
         <v>150</v>
@@ -3900,10 +4053,10 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="C103" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D103" t="s">
         <v>150</v>
@@ -3917,10 +4070,10 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="C104" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="D104" t="s">
         <v>150</v>
@@ -3934,10 +4087,10 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>556</v>
+        <v>205</v>
       </c>
       <c r="C105" t="s">
-        <v>557</v>
+        <v>206</v>
       </c>
       <c r="D105" t="s">
         <v>150</v>
@@ -3951,16 +4104,16 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="C106" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="D106" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E106" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">
@@ -3968,16 +4121,16 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="C107" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="D107" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E107" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.3">
@@ -3985,16 +4138,16 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="C108" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="D108" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E108" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.3">
@@ -4002,16 +4155,16 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>220</v>
+        <v>556</v>
       </c>
       <c r="C109" t="s">
-        <v>221</v>
+        <v>557</v>
       </c>
       <c r="D109" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E109" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
@@ -4019,16 +4172,16 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>222</v>
+        <v>587</v>
       </c>
       <c r="C110" t="s">
-        <v>223</v>
+        <v>588</v>
       </c>
       <c r="D110" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E110" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.3">
@@ -4036,16 +4189,16 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>224</v>
+        <v>589</v>
       </c>
       <c r="C111" t="s">
-        <v>225</v>
+        <v>590</v>
       </c>
       <c r="D111" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E111" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.3">
@@ -4053,16 +4206,16 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>226</v>
+        <v>591</v>
       </c>
       <c r="C112" t="s">
-        <v>227</v>
+        <v>592</v>
       </c>
       <c r="D112" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E112" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.3">
@@ -4070,16 +4223,16 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>228</v>
+        <v>593</v>
       </c>
       <c r="C113" t="s">
-        <v>229</v>
+        <v>594</v>
       </c>
       <c r="D113" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E113" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.3">
@@ -4087,16 +4240,16 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>230</v>
+        <v>595</v>
       </c>
       <c r="C114" t="s">
-        <v>231</v>
+        <v>596</v>
       </c>
       <c r="D114" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E114" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.3">
@@ -4104,16 +4257,16 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>232</v>
+        <v>597</v>
       </c>
       <c r="C115" t="s">
-        <v>233</v>
+        <v>598</v>
       </c>
       <c r="D115" t="s">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="E115" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.3">
@@ -4121,10 +4274,10 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>234</v>
+        <v>213</v>
       </c>
       <c r="C116" t="s">
-        <v>235</v>
+        <v>214</v>
       </c>
       <c r="D116" t="s">
         <v>215</v>
@@ -4138,10 +4291,10 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>236</v>
+        <v>216</v>
       </c>
       <c r="C117" t="s">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="D117" t="s">
         <v>215</v>
@@ -4155,10 +4308,10 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>238</v>
+        <v>218</v>
       </c>
       <c r="C118" t="s">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="D118" t="s">
         <v>215</v>
@@ -4172,10 +4325,10 @@
         <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C119" t="s">
-        <v>241</v>
+        <v>221</v>
       </c>
       <c r="D119" t="s">
         <v>215</v>
@@ -4189,10 +4342,10 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>242</v>
+        <v>222</v>
       </c>
       <c r="C120" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="D120" t="s">
         <v>215</v>
@@ -4206,10 +4359,10 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="C121" t="s">
-        <v>245</v>
+        <v>225</v>
       </c>
       <c r="D121" t="s">
         <v>215</v>
@@ -4223,10 +4376,10 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>246</v>
+        <v>226</v>
       </c>
       <c r="C122" t="s">
-        <v>247</v>
+        <v>227</v>
       </c>
       <c r="D122" t="s">
         <v>215</v>
@@ -4240,10 +4393,10 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>248</v>
+        <v>228</v>
       </c>
       <c r="C123" t="s">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="D123" t="s">
         <v>215</v>
@@ -4257,10 +4410,10 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="C124" t="s">
-        <v>251</v>
+        <v>231</v>
       </c>
       <c r="D124" t="s">
         <v>215</v>
@@ -4274,10 +4427,10 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>252</v>
+        <v>232</v>
       </c>
       <c r="C125" t="s">
-        <v>253</v>
+        <v>233</v>
       </c>
       <c r="D125" t="s">
         <v>215</v>
@@ -4291,10 +4444,10 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>254</v>
+        <v>234</v>
       </c>
       <c r="C126" t="s">
-        <v>255</v>
+        <v>235</v>
       </c>
       <c r="D126" t="s">
         <v>215</v>
@@ -4308,10 +4461,10 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
       <c r="C127" t="s">
-        <v>257</v>
+        <v>237</v>
       </c>
       <c r="D127" t="s">
         <v>215</v>
@@ -4325,10 +4478,10 @@
         <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="C128" t="s">
-        <v>259</v>
+        <v>239</v>
       </c>
       <c r="D128" t="s">
         <v>215</v>
@@ -4342,10 +4495,10 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="C129" t="s">
-        <v>261</v>
+        <v>241</v>
       </c>
       <c r="D129" t="s">
         <v>215</v>
@@ -4359,10 +4512,10 @@
         <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>262</v>
+        <v>242</v>
       </c>
       <c r="C130" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="D130" t="s">
         <v>215</v>
@@ -4376,10 +4529,10 @@
         <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>264</v>
+        <v>244</v>
       </c>
       <c r="C131" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
       <c r="D131" t="s">
         <v>215</v>
@@ -4393,10 +4546,10 @@
         <v>131</v>
       </c>
       <c r="B132" t="s">
-        <v>266</v>
+        <v>246</v>
       </c>
       <c r="C132" t="s">
-        <v>267</v>
+        <v>247</v>
       </c>
       <c r="D132" t="s">
         <v>215</v>
@@ -4410,10 +4563,10 @@
         <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>268</v>
+        <v>248</v>
       </c>
       <c r="C133" t="s">
-        <v>269</v>
+        <v>249</v>
       </c>
       <c r="D133" t="s">
         <v>215</v>
@@ -4427,10 +4580,10 @@
         <v>133</v>
       </c>
       <c r="B134" t="s">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C134" t="s">
-        <v>271</v>
+        <v>251</v>
       </c>
       <c r="D134" t="s">
         <v>215</v>
@@ -4444,10 +4597,10 @@
         <v>134</v>
       </c>
       <c r="B135" t="s">
-        <v>272</v>
+        <v>252</v>
       </c>
       <c r="C135" t="s">
-        <v>273</v>
+        <v>253</v>
       </c>
       <c r="D135" t="s">
         <v>215</v>
@@ -4461,10 +4614,10 @@
         <v>135</v>
       </c>
       <c r="B136" t="s">
-        <v>274</v>
+        <v>254</v>
       </c>
       <c r="C136" t="s">
-        <v>275</v>
+        <v>255</v>
       </c>
       <c r="D136" t="s">
         <v>215</v>
@@ -4478,10 +4631,10 @@
         <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>276</v>
+        <v>256</v>
       </c>
       <c r="C137" t="s">
-        <v>277</v>
+        <v>257</v>
       </c>
       <c r="D137" t="s">
         <v>215</v>
@@ -4495,10 +4648,10 @@
         <v>137</v>
       </c>
       <c r="B138" t="s">
-        <v>558</v>
+        <v>258</v>
       </c>
       <c r="C138" t="s">
-        <v>559</v>
+        <v>259</v>
       </c>
       <c r="D138" t="s">
         <v>215</v>
@@ -4512,13 +4665,13 @@
         <v>138</v>
       </c>
       <c r="B139" t="s">
-        <v>560</v>
+        <v>260</v>
       </c>
       <c r="C139" t="s">
-        <v>561</v>
+        <v>261</v>
       </c>
       <c r="D139" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E139" t="s">
         <v>10</v>
@@ -4529,16 +4682,16 @@
         <v>139</v>
       </c>
       <c r="B140" t="s">
-        <v>278</v>
+        <v>262</v>
       </c>
       <c r="C140" t="s">
-        <v>279</v>
+        <v>263</v>
       </c>
       <c r="D140" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E140" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.3">
@@ -4546,16 +4699,16 @@
         <v>140</v>
       </c>
       <c r="B141" t="s">
-        <v>280</v>
+        <v>264</v>
       </c>
       <c r="C141" t="s">
-        <v>281</v>
+        <v>265</v>
       </c>
       <c r="D141" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E141" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.3">
@@ -4563,16 +4716,16 @@
         <v>141</v>
       </c>
       <c r="B142" t="s">
-        <v>282</v>
+        <v>266</v>
       </c>
       <c r="C142" t="s">
-        <v>283</v>
+        <v>267</v>
       </c>
       <c r="D142" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E142" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.3">
@@ -4580,16 +4733,16 @@
         <v>142</v>
       </c>
       <c r="B143" t="s">
-        <v>284</v>
+        <v>268</v>
       </c>
       <c r="C143" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="D143" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E143" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.3">
@@ -4597,16 +4750,16 @@
         <v>143</v>
       </c>
       <c r="B144" t="s">
-        <v>286</v>
+        <v>270</v>
       </c>
       <c r="C144" t="s">
-        <v>287</v>
+        <v>271</v>
       </c>
       <c r="D144" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E144" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.3">
@@ -4614,16 +4767,16 @@
         <v>144</v>
       </c>
       <c r="B145" t="s">
-        <v>288</v>
+        <v>272</v>
       </c>
       <c r="C145" t="s">
-        <v>289</v>
+        <v>273</v>
       </c>
       <c r="D145" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E145" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.3">
@@ -4631,16 +4784,16 @@
         <v>145</v>
       </c>
       <c r="B146" t="s">
-        <v>290</v>
+        <v>274</v>
       </c>
       <c r="C146" t="s">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="D146" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E146" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.3">
@@ -4648,16 +4801,16 @@
         <v>146</v>
       </c>
       <c r="B147" t="s">
-        <v>292</v>
+        <v>276</v>
       </c>
       <c r="C147" t="s">
-        <v>293</v>
+        <v>277</v>
       </c>
       <c r="D147" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E147" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
@@ -4665,16 +4818,16 @@
         <v>147</v>
       </c>
       <c r="B148" t="s">
-        <v>294</v>
+        <v>558</v>
       </c>
       <c r="C148" t="s">
-        <v>295</v>
+        <v>559</v>
       </c>
       <c r="D148" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E148" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">
@@ -4682,16 +4835,16 @@
         <v>148</v>
       </c>
       <c r="B149" t="s">
-        <v>296</v>
+        <v>560</v>
       </c>
       <c r="C149" t="s">
-        <v>297</v>
+        <v>561</v>
       </c>
       <c r="D149" t="s">
         <v>4</v>
       </c>
       <c r="E149" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
@@ -4699,16 +4852,16 @@
         <v>149</v>
       </c>
       <c r="B150" t="s">
-        <v>298</v>
+        <v>599</v>
       </c>
       <c r="C150" t="s">
-        <v>299</v>
+        <v>600</v>
       </c>
       <c r="D150" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E150" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
@@ -4716,16 +4869,16 @@
         <v>150</v>
       </c>
       <c r="B151" t="s">
-        <v>300</v>
+        <v>601</v>
       </c>
       <c r="C151" t="s">
-        <v>301</v>
+        <v>602</v>
       </c>
       <c r="D151" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E151" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.3">
@@ -4733,16 +4886,16 @@
         <v>151</v>
       </c>
       <c r="B152" t="s">
-        <v>302</v>
+        <v>603</v>
       </c>
       <c r="C152" t="s">
-        <v>303</v>
+        <v>604</v>
       </c>
       <c r="D152" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E152" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.3">
@@ -4750,16 +4903,16 @@
         <v>152</v>
       </c>
       <c r="B153" t="s">
-        <v>304</v>
+        <v>605</v>
       </c>
       <c r="C153" t="s">
-        <v>305</v>
+        <v>606</v>
       </c>
       <c r="D153" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E153" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.3">
@@ -4767,16 +4920,16 @@
         <v>153</v>
       </c>
       <c r="B154" t="s">
-        <v>306</v>
+        <v>607</v>
       </c>
       <c r="C154" t="s">
-        <v>307</v>
+        <v>608</v>
       </c>
       <c r="D154" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E154" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.3">
@@ -4784,10 +4937,10 @@
         <v>154</v>
       </c>
       <c r="B155" t="s">
-        <v>308</v>
+        <v>278</v>
       </c>
       <c r="C155" t="s">
-        <v>309</v>
+        <v>279</v>
       </c>
       <c r="D155" t="s">
         <v>4</v>
@@ -4801,10 +4954,10 @@
         <v>155</v>
       </c>
       <c r="B156" t="s">
-        <v>310</v>
+        <v>280</v>
       </c>
       <c r="C156" t="s">
-        <v>311</v>
+        <v>281</v>
       </c>
       <c r="D156" t="s">
         <v>4</v>
@@ -4818,10 +4971,10 @@
         <v>156</v>
       </c>
       <c r="B157" t="s">
-        <v>312</v>
+        <v>282</v>
       </c>
       <c r="C157" t="s">
-        <v>313</v>
+        <v>283</v>
       </c>
       <c r="D157" t="s">
         <v>4</v>
@@ -4835,10 +4988,10 @@
         <v>157</v>
       </c>
       <c r="B158" t="s">
-        <v>314</v>
+        <v>284</v>
       </c>
       <c r="C158" t="s">
-        <v>315</v>
+        <v>285</v>
       </c>
       <c r="D158" t="s">
         <v>4</v>
@@ -4852,10 +5005,10 @@
         <v>158</v>
       </c>
       <c r="B159" t="s">
-        <v>316</v>
+        <v>286</v>
       </c>
       <c r="C159" t="s">
-        <v>317</v>
+        <v>287</v>
       </c>
       <c r="D159" t="s">
         <v>4</v>
@@ -4869,10 +5022,10 @@
         <v>159</v>
       </c>
       <c r="B160" t="s">
-        <v>318</v>
+        <v>288</v>
       </c>
       <c r="C160" t="s">
-        <v>319</v>
+        <v>289</v>
       </c>
       <c r="D160" t="s">
         <v>4</v>
@@ -4886,10 +5039,10 @@
         <v>160</v>
       </c>
       <c r="B161" t="s">
-        <v>320</v>
+        <v>290</v>
       </c>
       <c r="C161" t="s">
-        <v>321</v>
+        <v>291</v>
       </c>
       <c r="D161" t="s">
         <v>4</v>
@@ -4903,13 +5056,13 @@
         <v>161</v>
       </c>
       <c r="B162" t="s">
-        <v>322</v>
+        <v>292</v>
       </c>
       <c r="C162" t="s">
-        <v>323</v>
+        <v>293</v>
       </c>
       <c r="D162" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E162" t="s">
         <v>11</v>
@@ -4920,13 +5073,13 @@
         <v>162</v>
       </c>
       <c r="B163" t="s">
-        <v>324</v>
+        <v>294</v>
       </c>
       <c r="C163" t="s">
-        <v>325</v>
+        <v>295</v>
       </c>
       <c r="D163" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E163" t="s">
         <v>11</v>
@@ -4937,13 +5090,13 @@
         <v>163</v>
       </c>
       <c r="B164" t="s">
-        <v>326</v>
+        <v>296</v>
       </c>
       <c r="C164" t="s">
-        <v>327</v>
+        <v>297</v>
       </c>
       <c r="D164" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E164" t="s">
         <v>11</v>
@@ -4954,13 +5107,13 @@
         <v>164</v>
       </c>
       <c r="B165" t="s">
-        <v>328</v>
+        <v>298</v>
       </c>
       <c r="C165" t="s">
-        <v>329</v>
+        <v>299</v>
       </c>
       <c r="D165" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E165" t="s">
         <v>11</v>
@@ -4971,13 +5124,13 @@
         <v>165</v>
       </c>
       <c r="B166" t="s">
-        <v>330</v>
+        <v>300</v>
       </c>
       <c r="C166" t="s">
-        <v>331</v>
+        <v>301</v>
       </c>
       <c r="D166" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E166" t="s">
         <v>11</v>
@@ -4988,13 +5141,13 @@
         <v>166</v>
       </c>
       <c r="B167" t="s">
-        <v>332</v>
+        <v>302</v>
       </c>
       <c r="C167" t="s">
-        <v>333</v>
+        <v>303</v>
       </c>
       <c r="D167" t="s">
-        <v>150</v>
+        <v>4</v>
       </c>
       <c r="E167" t="s">
         <v>11</v>
@@ -5005,13 +5158,13 @@
         <v>167</v>
       </c>
       <c r="B168" t="s">
-        <v>334</v>
+        <v>304</v>
       </c>
       <c r="C168" t="s">
-        <v>335</v>
+        <v>305</v>
       </c>
       <c r="D168" t="s">
-        <v>215</v>
+        <v>4</v>
       </c>
       <c r="E168" t="s">
         <v>11</v>
@@ -5022,13 +5175,13 @@
         <v>168</v>
       </c>
       <c r="B169" t="s">
-        <v>336</v>
+        <v>306</v>
       </c>
       <c r="C169" t="s">
-        <v>337</v>
+        <v>307</v>
       </c>
       <c r="D169" t="s">
-        <v>215</v>
+        <v>4</v>
       </c>
       <c r="E169" t="s">
         <v>11</v>
@@ -5039,13 +5192,13 @@
         <v>169</v>
       </c>
       <c r="B170" t="s">
-        <v>338</v>
+        <v>308</v>
       </c>
       <c r="C170" t="s">
-        <v>339</v>
+        <v>309</v>
       </c>
       <c r="D170" t="s">
-        <v>215</v>
+        <v>4</v>
       </c>
       <c r="E170" t="s">
         <v>11</v>
@@ -5056,13 +5209,13 @@
         <v>170</v>
       </c>
       <c r="B171" t="s">
-        <v>340</v>
+        <v>310</v>
       </c>
       <c r="C171" t="s">
-        <v>341</v>
+        <v>311</v>
       </c>
       <c r="D171" t="s">
-        <v>215</v>
+        <v>4</v>
       </c>
       <c r="E171" t="s">
         <v>11</v>
@@ -5073,13 +5226,13 @@
         <v>171</v>
       </c>
       <c r="B172" t="s">
-        <v>342</v>
+        <v>312</v>
       </c>
       <c r="C172" t="s">
-        <v>343</v>
+        <v>313</v>
       </c>
       <c r="D172" t="s">
-        <v>215</v>
+        <v>4</v>
       </c>
       <c r="E172" t="s">
         <v>11</v>
@@ -5090,13 +5243,13 @@
         <v>172</v>
       </c>
       <c r="B173" t="s">
-        <v>344</v>
+        <v>314</v>
       </c>
       <c r="C173" t="s">
-        <v>345</v>
+        <v>315</v>
       </c>
       <c r="D173" t="s">
-        <v>215</v>
+        <v>4</v>
       </c>
       <c r="E173" t="s">
         <v>11</v>
@@ -5107,13 +5260,13 @@
         <v>173</v>
       </c>
       <c r="B174" t="s">
-        <v>346</v>
+        <v>316</v>
       </c>
       <c r="C174" t="s">
-        <v>347</v>
+        <v>317</v>
       </c>
       <c r="D174" t="s">
-        <v>215</v>
+        <v>4</v>
       </c>
       <c r="E174" t="s">
         <v>11</v>
@@ -5124,16 +5277,16 @@
         <v>174</v>
       </c>
       <c r="B175" t="s">
-        <v>348</v>
+        <v>318</v>
       </c>
       <c r="C175" t="s">
-        <v>349</v>
+        <v>319</v>
       </c>
       <c r="D175" t="s">
-        <v>350</v>
+        <v>4</v>
       </c>
       <c r="E175" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.3">
@@ -5141,16 +5294,16 @@
         <v>175</v>
       </c>
       <c r="B176" t="s">
-        <v>352</v>
+        <v>320</v>
       </c>
       <c r="C176" t="s">
-        <v>353</v>
+        <v>321</v>
       </c>
       <c r="D176" t="s">
-        <v>350</v>
+        <v>4</v>
       </c>
       <c r="E176" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.3">
@@ -5158,16 +5311,16 @@
         <v>176</v>
       </c>
       <c r="B177" t="s">
-        <v>354</v>
+        <v>322</v>
       </c>
       <c r="C177" t="s">
-        <v>355</v>
+        <v>323</v>
       </c>
       <c r="D177" t="s">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="E177" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.3">
@@ -5175,16 +5328,16 @@
         <v>177</v>
       </c>
       <c r="B178" t="s">
-        <v>356</v>
+        <v>324</v>
       </c>
       <c r="C178" t="s">
-        <v>357</v>
+        <v>325</v>
       </c>
       <c r="D178" t="s">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="E178" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.3">
@@ -5192,16 +5345,16 @@
         <v>178</v>
       </c>
       <c r="B179" t="s">
-        <v>358</v>
+        <v>326</v>
       </c>
       <c r="C179" t="s">
-        <v>359</v>
+        <v>327</v>
       </c>
       <c r="D179" t="s">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="E179" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.3">
@@ -5209,16 +5362,16 @@
         <v>179</v>
       </c>
       <c r="B180" t="s">
-        <v>360</v>
+        <v>328</v>
       </c>
       <c r="C180" t="s">
-        <v>361</v>
+        <v>329</v>
       </c>
       <c r="D180" t="s">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="E180" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.3">
@@ -5226,16 +5379,16 @@
         <v>180</v>
       </c>
       <c r="B181" t="s">
-        <v>362</v>
+        <v>330</v>
       </c>
       <c r="C181" t="s">
-        <v>363</v>
+        <v>331</v>
       </c>
       <c r="D181" t="s">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="E181" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.3">
@@ -5243,16 +5396,16 @@
         <v>181</v>
       </c>
       <c r="B182" t="s">
-        <v>364</v>
+        <v>332</v>
       </c>
       <c r="C182" t="s">
-        <v>365</v>
+        <v>333</v>
       </c>
       <c r="D182" t="s">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="E182" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.3">
@@ -5260,16 +5413,16 @@
         <v>182</v>
       </c>
       <c r="B183" t="s">
-        <v>366</v>
+        <v>334</v>
       </c>
       <c r="C183" t="s">
-        <v>367</v>
+        <v>335</v>
       </c>
       <c r="D183" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E183" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.3">
@@ -5277,16 +5430,16 @@
         <v>183</v>
       </c>
       <c r="B184" t="s">
-        <v>368</v>
+        <v>336</v>
       </c>
       <c r="C184" t="s">
-        <v>369</v>
+        <v>337</v>
       </c>
       <c r="D184" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E184" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.3">
@@ -5294,16 +5447,16 @@
         <v>184</v>
       </c>
       <c r="B185" t="s">
-        <v>370</v>
+        <v>338</v>
       </c>
       <c r="C185" t="s">
-        <v>371</v>
+        <v>339</v>
       </c>
       <c r="D185" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E185" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.3">
@@ -5311,16 +5464,16 @@
         <v>185</v>
       </c>
       <c r="B186" t="s">
-        <v>372</v>
+        <v>340</v>
       </c>
       <c r="C186" t="s">
-        <v>373</v>
+        <v>341</v>
       </c>
       <c r="D186" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E186" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.3">
@@ -5328,16 +5481,16 @@
         <v>186</v>
       </c>
       <c r="B187" t="s">
-        <v>374</v>
+        <v>342</v>
       </c>
       <c r="C187" t="s">
-        <v>375</v>
+        <v>343</v>
       </c>
       <c r="D187" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E187" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.3">
@@ -5345,16 +5498,16 @@
         <v>187</v>
       </c>
       <c r="B188" t="s">
-        <v>376</v>
+        <v>344</v>
       </c>
       <c r="C188" t="s">
-        <v>377</v>
+        <v>345</v>
       </c>
       <c r="D188" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E188" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.3">
@@ -5362,16 +5515,16 @@
         <v>188</v>
       </c>
       <c r="B189" t="s">
-        <v>378</v>
+        <v>346</v>
       </c>
       <c r="C189" t="s">
-        <v>379</v>
+        <v>347</v>
       </c>
       <c r="D189" t="s">
-        <v>350</v>
+        <v>215</v>
       </c>
       <c r="E189" t="s">
-        <v>351</v>
+        <v>11</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.3">
@@ -5379,10 +5532,10 @@
         <v>189</v>
       </c>
       <c r="B190" t="s">
-        <v>380</v>
+        <v>348</v>
       </c>
       <c r="C190" t="s">
-        <v>381</v>
+        <v>349</v>
       </c>
       <c r="D190" t="s">
         <v>350</v>
@@ -5396,10 +5549,10 @@
         <v>190</v>
       </c>
       <c r="B191" t="s">
-        <v>382</v>
+        <v>352</v>
       </c>
       <c r="C191" t="s">
-        <v>383</v>
+        <v>353</v>
       </c>
       <c r="D191" t="s">
         <v>350</v>
@@ -5413,10 +5566,10 @@
         <v>191</v>
       </c>
       <c r="B192" t="s">
-        <v>384</v>
+        <v>354</v>
       </c>
       <c r="C192" t="s">
-        <v>385</v>
+        <v>355</v>
       </c>
       <c r="D192" t="s">
         <v>350</v>
@@ -5430,10 +5583,10 @@
         <v>192</v>
       </c>
       <c r="B193" t="s">
-        <v>386</v>
+        <v>356</v>
       </c>
       <c r="C193" t="s">
-        <v>387</v>
+        <v>357</v>
       </c>
       <c r="D193" t="s">
         <v>350</v>
@@ -5447,10 +5600,10 @@
         <v>193</v>
       </c>
       <c r="B194" t="s">
-        <v>388</v>
+        <v>358</v>
       </c>
       <c r="C194" t="s">
-        <v>389</v>
+        <v>359</v>
       </c>
       <c r="D194" t="s">
         <v>350</v>
@@ -5464,10 +5617,10 @@
         <v>194</v>
       </c>
       <c r="B195" t="s">
-        <v>390</v>
+        <v>360</v>
       </c>
       <c r="C195" t="s">
-        <v>391</v>
+        <v>361</v>
       </c>
       <c r="D195" t="s">
         <v>350</v>
@@ -5481,10 +5634,10 @@
         <v>195</v>
       </c>
       <c r="B196" t="s">
-        <v>392</v>
+        <v>362</v>
       </c>
       <c r="C196" t="s">
-        <v>393</v>
+        <v>363</v>
       </c>
       <c r="D196" t="s">
         <v>350</v>
@@ -5498,10 +5651,10 @@
         <v>196</v>
       </c>
       <c r="B197" t="s">
-        <v>394</v>
+        <v>364</v>
       </c>
       <c r="C197" t="s">
-        <v>395</v>
+        <v>365</v>
       </c>
       <c r="D197" t="s">
         <v>350</v>
@@ -5515,10 +5668,10 @@
         <v>197</v>
       </c>
       <c r="B198" t="s">
-        <v>396</v>
+        <v>366</v>
       </c>
       <c r="C198" t="s">
-        <v>397</v>
+        <v>367</v>
       </c>
       <c r="D198" t="s">
         <v>350</v>
@@ -5532,10 +5685,10 @@
         <v>198</v>
       </c>
       <c r="B199" t="s">
-        <v>398</v>
+        <v>368</v>
       </c>
       <c r="C199" t="s">
-        <v>399</v>
+        <v>369</v>
       </c>
       <c r="D199" t="s">
         <v>350</v>
@@ -5549,10 +5702,10 @@
         <v>199</v>
       </c>
       <c r="B200" t="s">
-        <v>400</v>
+        <v>370</v>
       </c>
       <c r="C200" t="s">
-        <v>401</v>
+        <v>371</v>
       </c>
       <c r="D200" t="s">
         <v>350</v>
@@ -5566,10 +5719,10 @@
         <v>200</v>
       </c>
       <c r="B201" t="s">
-        <v>402</v>
+        <v>372</v>
       </c>
       <c r="C201" t="s">
-        <v>403</v>
+        <v>373</v>
       </c>
       <c r="D201" t="s">
         <v>350</v>
@@ -5583,10 +5736,10 @@
         <v>201</v>
       </c>
       <c r="B202" t="s">
-        <v>404</v>
+        <v>374</v>
       </c>
       <c r="C202" t="s">
-        <v>405</v>
+        <v>375</v>
       </c>
       <c r="D202" t="s">
         <v>350</v>
@@ -5600,10 +5753,10 @@
         <v>202</v>
       </c>
       <c r="B203" t="s">
-        <v>406</v>
+        <v>376</v>
       </c>
       <c r="C203" t="s">
-        <v>407</v>
+        <v>377</v>
       </c>
       <c r="D203" t="s">
         <v>350</v>
@@ -5617,10 +5770,10 @@
         <v>203</v>
       </c>
       <c r="B204" t="s">
-        <v>408</v>
+        <v>378</v>
       </c>
       <c r="C204" t="s">
-        <v>409</v>
+        <v>379</v>
       </c>
       <c r="D204" t="s">
         <v>350</v>
@@ -5634,10 +5787,10 @@
         <v>204</v>
       </c>
       <c r="B205" t="s">
-        <v>410</v>
+        <v>380</v>
       </c>
       <c r="C205" t="s">
-        <v>411</v>
+        <v>381</v>
       </c>
       <c r="D205" t="s">
         <v>350</v>
@@ -5651,10 +5804,10 @@
         <v>205</v>
       </c>
       <c r="B206" t="s">
-        <v>412</v>
+        <v>382</v>
       </c>
       <c r="C206" t="s">
-        <v>413</v>
+        <v>383</v>
       </c>
       <c r="D206" t="s">
         <v>350</v>
@@ -5668,16 +5821,16 @@
         <v>206</v>
       </c>
       <c r="B207" t="s">
-        <v>414</v>
+        <v>384</v>
       </c>
       <c r="C207" t="s">
-        <v>415</v>
+        <v>385</v>
       </c>
       <c r="D207" t="s">
         <v>350</v>
       </c>
       <c r="E207" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.3">
@@ -5685,16 +5838,16 @@
         <v>207</v>
       </c>
       <c r="B208" t="s">
-        <v>417</v>
+        <v>386</v>
       </c>
       <c r="C208" t="s">
-        <v>418</v>
+        <v>387</v>
       </c>
       <c r="D208" t="s">
         <v>350</v>
       </c>
       <c r="E208" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.3">
@@ -5702,16 +5855,16 @@
         <v>208</v>
       </c>
       <c r="B209" t="s">
-        <v>419</v>
+        <v>388</v>
       </c>
       <c r="C209" t="s">
-        <v>420</v>
+        <v>389</v>
       </c>
       <c r="D209" t="s">
         <v>350</v>
       </c>
       <c r="E209" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.3">
@@ -5719,16 +5872,16 @@
         <v>209</v>
       </c>
       <c r="B210" t="s">
-        <v>421</v>
+        <v>390</v>
       </c>
       <c r="C210" t="s">
-        <v>422</v>
+        <v>391</v>
       </c>
       <c r="D210" t="s">
         <v>350</v>
       </c>
       <c r="E210" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.3">
@@ -5736,16 +5889,16 @@
         <v>210</v>
       </c>
       <c r="B211" t="s">
-        <v>423</v>
+        <v>392</v>
       </c>
       <c r="C211" t="s">
-        <v>424</v>
+        <v>393</v>
       </c>
       <c r="D211" t="s">
         <v>350</v>
       </c>
       <c r="E211" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.3">
@@ -5753,16 +5906,16 @@
         <v>211</v>
       </c>
       <c r="B212" t="s">
-        <v>425</v>
+        <v>394</v>
       </c>
       <c r="C212" t="s">
-        <v>426</v>
+        <v>395</v>
       </c>
       <c r="D212" t="s">
         <v>350</v>
       </c>
       <c r="E212" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.3">
@@ -5770,16 +5923,16 @@
         <v>212</v>
       </c>
       <c r="B213" t="s">
-        <v>427</v>
+        <v>396</v>
       </c>
       <c r="C213" t="s">
-        <v>428</v>
+        <v>397</v>
       </c>
       <c r="D213" t="s">
         <v>350</v>
       </c>
       <c r="E213" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.3">
@@ -5787,16 +5940,16 @@
         <v>213</v>
       </c>
       <c r="B214" t="s">
-        <v>429</v>
+        <v>398</v>
       </c>
       <c r="C214" t="s">
-        <v>430</v>
+        <v>399</v>
       </c>
       <c r="D214" t="s">
         <v>350</v>
       </c>
       <c r="E214" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.3">
@@ -5804,16 +5957,16 @@
         <v>214</v>
       </c>
       <c r="B215" t="s">
-        <v>431</v>
+        <v>400</v>
       </c>
       <c r="C215" t="s">
-        <v>432</v>
+        <v>401</v>
       </c>
       <c r="D215" t="s">
         <v>350</v>
       </c>
       <c r="E215" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="216" spans="1:5" x14ac:dyDescent="0.3">
@@ -5821,16 +5974,16 @@
         <v>215</v>
       </c>
       <c r="B216" t="s">
-        <v>433</v>
+        <v>402</v>
       </c>
       <c r="C216" t="s">
-        <v>434</v>
+        <v>403</v>
       </c>
       <c r="D216" t="s">
         <v>350</v>
       </c>
       <c r="E216" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.3">
@@ -5838,16 +5991,16 @@
         <v>216</v>
       </c>
       <c r="B217" t="s">
-        <v>435</v>
+        <v>404</v>
       </c>
       <c r="C217" t="s">
-        <v>436</v>
+        <v>405</v>
       </c>
       <c r="D217" t="s">
         <v>350</v>
       </c>
       <c r="E217" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="218" spans="1:5" x14ac:dyDescent="0.3">
@@ -5855,16 +6008,16 @@
         <v>217</v>
       </c>
       <c r="B218" t="s">
-        <v>437</v>
+        <v>406</v>
       </c>
       <c r="C218" t="s">
-        <v>438</v>
+        <v>407</v>
       </c>
       <c r="D218" t="s">
         <v>350</v>
       </c>
       <c r="E218" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.3">
@@ -5872,16 +6025,16 @@
         <v>218</v>
       </c>
       <c r="B219" t="s">
-        <v>439</v>
+        <v>408</v>
       </c>
       <c r="C219" t="s">
-        <v>440</v>
+        <v>409</v>
       </c>
       <c r="D219" t="s">
         <v>350</v>
       </c>
       <c r="E219" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.3">
@@ -5889,16 +6042,16 @@
         <v>219</v>
       </c>
       <c r="B220" t="s">
-        <v>441</v>
+        <v>410</v>
       </c>
       <c r="C220" t="s">
-        <v>442</v>
+        <v>411</v>
       </c>
       <c r="D220" t="s">
-        <v>443</v>
+        <v>350</v>
       </c>
       <c r="E220" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.3">
@@ -5906,16 +6059,16 @@
         <v>220</v>
       </c>
       <c r="B221" t="s">
-        <v>444</v>
+        <v>412</v>
       </c>
       <c r="C221" t="s">
-        <v>445</v>
+        <v>413</v>
       </c>
       <c r="D221" t="s">
-        <v>443</v>
+        <v>350</v>
       </c>
       <c r="E221" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.3">
@@ -5923,16 +6076,16 @@
         <v>221</v>
       </c>
       <c r="B222" t="s">
-        <v>446</v>
+        <v>609</v>
       </c>
       <c r="C222" t="s">
-        <v>447</v>
+        <v>610</v>
       </c>
       <c r="D222" t="s">
         <v>3</v>
       </c>
       <c r="E222" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.3">
@@ -5940,16 +6093,16 @@
         <v>222</v>
       </c>
       <c r="B223" t="s">
-        <v>448</v>
+        <v>611</v>
       </c>
       <c r="C223" t="s">
-        <v>449</v>
+        <v>612</v>
       </c>
       <c r="D223" t="s">
-        <v>3</v>
+        <v>443</v>
       </c>
       <c r="E223" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.3">
@@ -5957,16 +6110,16 @@
         <v>223</v>
       </c>
       <c r="B224" t="s">
-        <v>450</v>
+        <v>552</v>
       </c>
       <c r="C224" t="s">
-        <v>451</v>
+        <v>613</v>
       </c>
       <c r="D224" t="s">
-        <v>3</v>
+        <v>131</v>
       </c>
       <c r="E224" t="s">
-        <v>416</v>
+        <v>351</v>
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.3">
@@ -5974,13 +6127,13 @@
         <v>224</v>
       </c>
       <c r="B225" t="s">
-        <v>452</v>
+        <v>414</v>
       </c>
       <c r="C225" t="s">
-        <v>453</v>
+        <v>415</v>
       </c>
       <c r="D225" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E225" t="s">
         <v>416</v>
@@ -5991,13 +6144,13 @@
         <v>225</v>
       </c>
       <c r="B226" t="s">
-        <v>454</v>
+        <v>417</v>
       </c>
       <c r="C226" t="s">
-        <v>455</v>
+        <v>418</v>
       </c>
       <c r="D226" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E226" t="s">
         <v>416</v>
@@ -6008,13 +6161,13 @@
         <v>226</v>
       </c>
       <c r="B227" t="s">
-        <v>456</v>
+        <v>419</v>
       </c>
       <c r="C227" t="s">
-        <v>457</v>
+        <v>420</v>
       </c>
       <c r="D227" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E227" t="s">
         <v>416</v>
@@ -6025,13 +6178,13 @@
         <v>227</v>
       </c>
       <c r="B228" t="s">
-        <v>458</v>
+        <v>421</v>
       </c>
       <c r="C228" t="s">
-        <v>459</v>
+        <v>422</v>
       </c>
       <c r="D228" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E228" t="s">
         <v>416</v>
@@ -6042,13 +6195,13 @@
         <v>228</v>
       </c>
       <c r="B229" t="s">
-        <v>460</v>
+        <v>423</v>
       </c>
       <c r="C229" t="s">
-        <v>461</v>
+        <v>424</v>
       </c>
       <c r="D229" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E229" t="s">
         <v>416</v>
@@ -6059,13 +6212,13 @@
         <v>229</v>
       </c>
       <c r="B230" t="s">
-        <v>462</v>
+        <v>425</v>
       </c>
       <c r="C230" t="s">
-        <v>463</v>
+        <v>426</v>
       </c>
       <c r="D230" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E230" t="s">
         <v>416</v>
@@ -6076,13 +6229,13 @@
         <v>230</v>
       </c>
       <c r="B231" t="s">
-        <v>464</v>
+        <v>427</v>
       </c>
       <c r="C231" t="s">
-        <v>465</v>
+        <v>428</v>
       </c>
       <c r="D231" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E231" t="s">
         <v>416</v>
@@ -6093,13 +6246,13 @@
         <v>231</v>
       </c>
       <c r="B232" t="s">
-        <v>562</v>
+        <v>429</v>
       </c>
       <c r="C232" t="s">
-        <v>563</v>
+        <v>430</v>
       </c>
       <c r="D232" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E232" t="s">
         <v>416</v>
@@ -6110,13 +6263,13 @@
         <v>232</v>
       </c>
       <c r="B233" t="s">
-        <v>466</v>
+        <v>431</v>
       </c>
       <c r="C233" t="s">
-        <v>467</v>
+        <v>432</v>
       </c>
       <c r="D233" t="s">
-        <v>468</v>
+        <v>350</v>
       </c>
       <c r="E233" t="s">
         <v>416</v>
@@ -6127,13 +6280,13 @@
         <v>233</v>
       </c>
       <c r="B234" t="s">
-        <v>469</v>
+        <v>433</v>
       </c>
       <c r="C234" t="s">
-        <v>470</v>
+        <v>434</v>
       </c>
       <c r="D234" t="s">
-        <v>468</v>
+        <v>350</v>
       </c>
       <c r="E234" t="s">
         <v>416</v>
@@ -6144,13 +6297,13 @@
         <v>234</v>
       </c>
       <c r="B235" t="s">
-        <v>471</v>
+        <v>435</v>
       </c>
       <c r="C235" t="s">
-        <v>472</v>
+        <v>436</v>
       </c>
       <c r="D235" t="s">
-        <v>468</v>
+        <v>350</v>
       </c>
       <c r="E235" t="s">
         <v>416</v>
@@ -6161,13 +6314,13 @@
         <v>235</v>
       </c>
       <c r="B236" t="s">
-        <v>473</v>
+        <v>437</v>
       </c>
       <c r="C236" t="s">
-        <v>474</v>
+        <v>438</v>
       </c>
       <c r="D236" t="s">
-        <v>468</v>
+        <v>350</v>
       </c>
       <c r="E236" t="s">
         <v>416</v>
@@ -6178,13 +6331,13 @@
         <v>236</v>
       </c>
       <c r="B237" t="s">
-        <v>475</v>
+        <v>439</v>
       </c>
       <c r="C237" t="s">
-        <v>476</v>
+        <v>440</v>
       </c>
       <c r="D237" t="s">
-        <v>468</v>
+        <v>350</v>
       </c>
       <c r="E237" t="s">
         <v>416</v>
@@ -6195,13 +6348,13 @@
         <v>237</v>
       </c>
       <c r="B238" t="s">
-        <v>477</v>
+        <v>441</v>
       </c>
       <c r="C238" t="s">
-        <v>478</v>
+        <v>442</v>
       </c>
       <c r="D238" t="s">
-        <v>468</v>
+        <v>443</v>
       </c>
       <c r="E238" t="s">
         <v>416</v>
@@ -6212,13 +6365,13 @@
         <v>238</v>
       </c>
       <c r="B239" t="s">
-        <v>479</v>
+        <v>444</v>
       </c>
       <c r="C239" t="s">
-        <v>480</v>
+        <v>445</v>
       </c>
       <c r="D239" t="s">
-        <v>468</v>
+        <v>443</v>
       </c>
       <c r="E239" t="s">
         <v>416</v>
@@ -6229,13 +6382,13 @@
         <v>239</v>
       </c>
       <c r="B240" t="s">
-        <v>481</v>
+        <v>446</v>
       </c>
       <c r="C240" t="s">
-        <v>482</v>
+        <v>447</v>
       </c>
       <c r="D240" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E240" t="s">
         <v>416</v>
@@ -6246,13 +6399,13 @@
         <v>240</v>
       </c>
       <c r="B241" t="s">
-        <v>483</v>
+        <v>448</v>
       </c>
       <c r="C241" t="s">
-        <v>484</v>
+        <v>449</v>
       </c>
       <c r="D241" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E241" t="s">
         <v>416</v>
@@ -6263,16 +6416,16 @@
         <v>241</v>
       </c>
       <c r="B242" t="s">
-        <v>485</v>
+        <v>450</v>
       </c>
       <c r="C242" t="s">
-        <v>486</v>
+        <v>451</v>
       </c>
       <c r="D242" t="s">
-        <v>487</v>
+        <v>3</v>
       </c>
       <c r="E242" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="243" spans="1:5" x14ac:dyDescent="0.3">
@@ -6280,16 +6433,16 @@
         <v>242</v>
       </c>
       <c r="B243" t="s">
-        <v>489</v>
+        <v>452</v>
       </c>
       <c r="C243" t="s">
-        <v>490</v>
+        <v>453</v>
       </c>
       <c r="D243" t="s">
-        <v>487</v>
+        <v>3</v>
       </c>
       <c r="E243" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="244" spans="1:5" x14ac:dyDescent="0.3">
@@ -6297,16 +6450,16 @@
         <v>243</v>
       </c>
       <c r="B244" t="s">
-        <v>491</v>
+        <v>454</v>
       </c>
       <c r="C244" t="s">
-        <v>492</v>
+        <v>455</v>
       </c>
       <c r="D244" t="s">
-        <v>487</v>
+        <v>3</v>
       </c>
       <c r="E244" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="245" spans="1:5" x14ac:dyDescent="0.3">
@@ -6314,16 +6467,16 @@
         <v>244</v>
       </c>
       <c r="B245" t="s">
-        <v>493</v>
+        <v>456</v>
       </c>
       <c r="C245" t="s">
-        <v>494</v>
+        <v>457</v>
       </c>
       <c r="D245" t="s">
-        <v>487</v>
+        <v>3</v>
       </c>
       <c r="E245" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="246" spans="1:5" x14ac:dyDescent="0.3">
@@ -6331,16 +6484,16 @@
         <v>245</v>
       </c>
       <c r="B246" t="s">
-        <v>495</v>
+        <v>458</v>
       </c>
       <c r="C246" t="s">
-        <v>496</v>
+        <v>459</v>
       </c>
       <c r="D246" t="s">
-        <v>487</v>
+        <v>3</v>
       </c>
       <c r="E246" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="247" spans="1:5" x14ac:dyDescent="0.3">
@@ -6348,16 +6501,16 @@
         <v>246</v>
       </c>
       <c r="B247" t="s">
-        <v>497</v>
+        <v>460</v>
       </c>
       <c r="C247" t="s">
-        <v>498</v>
+        <v>461</v>
       </c>
       <c r="D247" t="s">
-        <v>487</v>
+        <v>3</v>
       </c>
       <c r="E247" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="248" spans="1:5" x14ac:dyDescent="0.3">
@@ -6365,16 +6518,16 @@
         <v>247</v>
       </c>
       <c r="B248" t="s">
-        <v>499</v>
+        <v>462</v>
       </c>
       <c r="C248" t="s">
-        <v>500</v>
+        <v>463</v>
       </c>
       <c r="D248" t="s">
-        <v>487</v>
+        <v>3</v>
       </c>
       <c r="E248" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="249" spans="1:5" x14ac:dyDescent="0.3">
@@ -6382,16 +6535,16 @@
         <v>248</v>
       </c>
       <c r="B249" t="s">
-        <v>501</v>
+        <v>464</v>
       </c>
       <c r="C249" t="s">
-        <v>502</v>
+        <v>465</v>
       </c>
       <c r="D249" t="s">
-        <v>487</v>
+        <v>3</v>
       </c>
       <c r="E249" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="250" spans="1:5" x14ac:dyDescent="0.3">
@@ -6399,16 +6552,16 @@
         <v>249</v>
       </c>
       <c r="B250" t="s">
-        <v>503</v>
+        <v>562</v>
       </c>
       <c r="C250" t="s">
-        <v>504</v>
+        <v>563</v>
       </c>
       <c r="D250" t="s">
-        <v>487</v>
+        <v>3</v>
       </c>
       <c r="E250" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="251" spans="1:5" x14ac:dyDescent="0.3">
@@ -6416,16 +6569,16 @@
         <v>250</v>
       </c>
       <c r="B251" t="s">
-        <v>505</v>
+        <v>466</v>
       </c>
       <c r="C251" t="s">
-        <v>506</v>
+        <v>467</v>
       </c>
       <c r="D251" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E251" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="252" spans="1:5" x14ac:dyDescent="0.3">
@@ -6433,16 +6586,16 @@
         <v>251</v>
       </c>
       <c r="B252" t="s">
-        <v>564</v>
+        <v>469</v>
       </c>
       <c r="C252" t="s">
-        <v>565</v>
+        <v>470</v>
       </c>
       <c r="D252" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E252" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="253" spans="1:5" x14ac:dyDescent="0.3">
@@ -6450,16 +6603,16 @@
         <v>252</v>
       </c>
       <c r="B253" t="s">
-        <v>566</v>
+        <v>471</v>
       </c>
       <c r="C253" t="s">
-        <v>567</v>
+        <v>472</v>
       </c>
       <c r="D253" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E253" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="254" spans="1:5" x14ac:dyDescent="0.3">
@@ -6467,16 +6620,16 @@
         <v>253</v>
       </c>
       <c r="B254" t="s">
-        <v>507</v>
+        <v>473</v>
       </c>
       <c r="C254" t="s">
-        <v>508</v>
+        <v>474</v>
       </c>
       <c r="D254" t="s">
-        <v>509</v>
+        <v>468</v>
       </c>
       <c r="E254" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="255" spans="1:5" x14ac:dyDescent="0.3">
@@ -6484,16 +6637,16 @@
         <v>254</v>
       </c>
       <c r="B255" t="s">
-        <v>510</v>
+        <v>475</v>
       </c>
       <c r="C255" t="s">
-        <v>511</v>
+        <v>476</v>
       </c>
       <c r="D255" t="s">
-        <v>509</v>
+        <v>468</v>
       </c>
       <c r="E255" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="256" spans="1:5" x14ac:dyDescent="0.3">
@@ -6501,16 +6654,16 @@
         <v>255</v>
       </c>
       <c r="B256" t="s">
-        <v>512</v>
+        <v>477</v>
       </c>
       <c r="C256" t="s">
-        <v>513</v>
+        <v>478</v>
       </c>
       <c r="D256" t="s">
-        <v>514</v>
+        <v>468</v>
       </c>
       <c r="E256" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="257" spans="1:5" x14ac:dyDescent="0.3">
@@ -6518,16 +6671,16 @@
         <v>256</v>
       </c>
       <c r="B257" t="s">
-        <v>515</v>
+        <v>479</v>
       </c>
       <c r="C257" t="s">
-        <v>516</v>
+        <v>480</v>
       </c>
       <c r="D257" t="s">
-        <v>514</v>
+        <v>468</v>
       </c>
       <c r="E257" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="258" spans="1:5" x14ac:dyDescent="0.3">
@@ -6535,16 +6688,16 @@
         <v>257</v>
       </c>
       <c r="B258" t="s">
-        <v>517</v>
+        <v>481</v>
       </c>
       <c r="C258" t="s">
-        <v>518</v>
+        <v>482</v>
       </c>
       <c r="D258" t="s">
-        <v>514</v>
+        <v>468</v>
       </c>
       <c r="E258" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="259" spans="1:5" x14ac:dyDescent="0.3">
@@ -6552,16 +6705,16 @@
         <v>258</v>
       </c>
       <c r="B259" t="s">
-        <v>519</v>
+        <v>483</v>
       </c>
       <c r="C259" t="s">
-        <v>520</v>
+        <v>484</v>
       </c>
       <c r="D259" t="s">
-        <v>521</v>
+        <v>468</v>
       </c>
       <c r="E259" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="260" spans="1:5" x14ac:dyDescent="0.3">
@@ -6569,16 +6722,16 @@
         <v>259</v>
       </c>
       <c r="B260" t="s">
-        <v>522</v>
+        <v>614</v>
       </c>
       <c r="C260" t="s">
-        <v>523</v>
+        <v>615</v>
       </c>
       <c r="D260" t="s">
-        <v>521</v>
+        <v>468</v>
       </c>
       <c r="E260" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="261" spans="1:5" x14ac:dyDescent="0.3">
@@ -6586,16 +6739,16 @@
         <v>260</v>
       </c>
       <c r="B261" t="s">
-        <v>568</v>
+        <v>616</v>
       </c>
       <c r="C261" t="s">
-        <v>569</v>
+        <v>617</v>
       </c>
       <c r="D261" t="s">
-        <v>521</v>
+        <v>543</v>
       </c>
       <c r="E261" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="262" spans="1:5" x14ac:dyDescent="0.3">
@@ -6603,16 +6756,16 @@
         <v>261</v>
       </c>
       <c r="B262" t="s">
-        <v>570</v>
+        <v>618</v>
       </c>
       <c r="C262" t="s">
-        <v>571</v>
+        <v>619</v>
       </c>
       <c r="D262" t="s">
-        <v>521</v>
+        <v>487</v>
       </c>
       <c r="E262" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="263" spans="1:5" x14ac:dyDescent="0.3">
@@ -6620,16 +6773,16 @@
         <v>262</v>
       </c>
       <c r="B263" t="s">
-        <v>524</v>
+        <v>620</v>
       </c>
       <c r="C263" t="s">
-        <v>525</v>
+        <v>621</v>
       </c>
       <c r="D263" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="E263" t="s">
-        <v>488</v>
+        <v>416</v>
       </c>
     </row>
     <row r="264" spans="1:5" x14ac:dyDescent="0.3">
@@ -6637,13 +6790,13 @@
         <v>263</v>
       </c>
       <c r="B264" t="s">
-        <v>527</v>
+        <v>485</v>
       </c>
       <c r="C264" t="s">
-        <v>528</v>
+        <v>486</v>
       </c>
       <c r="D264" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="E264" t="s">
         <v>488</v>
@@ -6654,13 +6807,13 @@
         <v>264</v>
       </c>
       <c r="B265" t="s">
-        <v>529</v>
+        <v>489</v>
       </c>
       <c r="C265" t="s">
-        <v>530</v>
+        <v>490</v>
       </c>
       <c r="D265" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="E265" t="s">
         <v>488</v>
@@ -6671,13 +6824,13 @@
         <v>265</v>
       </c>
       <c r="B266" t="s">
-        <v>531</v>
+        <v>491</v>
       </c>
       <c r="C266" t="s">
-        <v>532</v>
+        <v>492</v>
       </c>
       <c r="D266" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="E266" t="s">
         <v>488</v>
@@ -6688,13 +6841,13 @@
         <v>266</v>
       </c>
       <c r="B267" t="s">
-        <v>533</v>
+        <v>493</v>
       </c>
       <c r="C267" t="s">
-        <v>534</v>
+        <v>494</v>
       </c>
       <c r="D267" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="E267" t="s">
         <v>488</v>
@@ -6705,13 +6858,13 @@
         <v>267</v>
       </c>
       <c r="B268" t="s">
-        <v>535</v>
+        <v>495</v>
       </c>
       <c r="C268" t="s">
-        <v>536</v>
+        <v>496</v>
       </c>
       <c r="D268" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="E268" t="s">
         <v>488</v>
@@ -6722,13 +6875,13 @@
         <v>268</v>
       </c>
       <c r="B269" t="s">
-        <v>537</v>
+        <v>497</v>
       </c>
       <c r="C269" t="s">
-        <v>538</v>
+        <v>498</v>
       </c>
       <c r="D269" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="E269" t="s">
         <v>488</v>
@@ -6739,13 +6892,13 @@
         <v>269</v>
       </c>
       <c r="B270" t="s">
-        <v>539</v>
+        <v>499</v>
       </c>
       <c r="C270" t="s">
-        <v>540</v>
+        <v>500</v>
       </c>
       <c r="D270" t="s">
-        <v>526</v>
+        <v>487</v>
       </c>
       <c r="E270" t="s">
         <v>488</v>
@@ -6756,13 +6909,13 @@
         <v>270</v>
       </c>
       <c r="B271" t="s">
-        <v>541</v>
+        <v>501</v>
       </c>
       <c r="C271" t="s">
-        <v>542</v>
+        <v>502</v>
       </c>
       <c r="D271" t="s">
-        <v>543</v>
+        <v>487</v>
       </c>
       <c r="E271" t="s">
         <v>488</v>
@@ -6773,13 +6926,13 @@
         <v>271</v>
       </c>
       <c r="B272" t="s">
-        <v>544</v>
+        <v>503</v>
       </c>
       <c r="C272" t="s">
-        <v>545</v>
+        <v>504</v>
       </c>
       <c r="D272" t="s">
-        <v>543</v>
+        <v>487</v>
       </c>
       <c r="E272" t="s">
         <v>488</v>
@@ -6790,13 +6943,13 @@
         <v>272</v>
       </c>
       <c r="B273" t="s">
-        <v>546</v>
+        <v>505</v>
       </c>
       <c r="C273" t="s">
-        <v>547</v>
+        <v>506</v>
       </c>
       <c r="D273" t="s">
-        <v>543</v>
+        <v>487</v>
       </c>
       <c r="E273" t="s">
         <v>488</v>
@@ -6807,13 +6960,13 @@
         <v>273</v>
       </c>
       <c r="B274" t="s">
-        <v>572</v>
+        <v>564</v>
       </c>
       <c r="C274" t="s">
-        <v>573</v>
+        <v>565</v>
       </c>
       <c r="D274" t="s">
-        <v>350</v>
+        <v>487</v>
       </c>
       <c r="E274" t="s">
         <v>488</v>
@@ -6824,13 +6977,13 @@
         <v>274</v>
       </c>
       <c r="B275" t="s">
-        <v>574</v>
+        <v>566</v>
       </c>
       <c r="C275" t="s">
-        <v>575</v>
+        <v>567</v>
       </c>
       <c r="D275" t="s">
-        <v>468</v>
+        <v>487</v>
       </c>
       <c r="E275" t="s">
         <v>488</v>
@@ -6841,15 +6994,457 @@
         <v>275</v>
       </c>
       <c r="B276" t="s">
+        <v>507</v>
+      </c>
+      <c r="C276" t="s">
+        <v>508</v>
+      </c>
+      <c r="D276" t="s">
+        <v>509</v>
+      </c>
+      <c r="E276" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="277" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A277">
+        <v>276</v>
+      </c>
+      <c r="B277" t="s">
+        <v>510</v>
+      </c>
+      <c r="C277" t="s">
+        <v>511</v>
+      </c>
+      <c r="D277" t="s">
+        <v>509</v>
+      </c>
+      <c r="E277" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="278" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A278">
+        <v>277</v>
+      </c>
+      <c r="B278" t="s">
+        <v>512</v>
+      </c>
+      <c r="C278" t="s">
+        <v>513</v>
+      </c>
+      <c r="D278" t="s">
+        <v>514</v>
+      </c>
+      <c r="E278" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="279" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A279">
+        <v>278</v>
+      </c>
+      <c r="B279" t="s">
+        <v>515</v>
+      </c>
+      <c r="C279" t="s">
+        <v>516</v>
+      </c>
+      <c r="D279" t="s">
+        <v>514</v>
+      </c>
+      <c r="E279" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="280" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A280">
+        <v>279</v>
+      </c>
+      <c r="B280" t="s">
+        <v>517</v>
+      </c>
+      <c r="C280" t="s">
+        <v>518</v>
+      </c>
+      <c r="D280" t="s">
+        <v>514</v>
+      </c>
+      <c r="E280" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="281" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A281">
+        <v>280</v>
+      </c>
+      <c r="B281" t="s">
+        <v>519</v>
+      </c>
+      <c r="C281" t="s">
+        <v>520</v>
+      </c>
+      <c r="D281" t="s">
+        <v>521</v>
+      </c>
+      <c r="E281" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="282" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A282">
+        <v>281</v>
+      </c>
+      <c r="B282" t="s">
+        <v>522</v>
+      </c>
+      <c r="C282" t="s">
+        <v>523</v>
+      </c>
+      <c r="D282" t="s">
+        <v>521</v>
+      </c>
+      <c r="E282" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="283" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A283">
+        <v>282</v>
+      </c>
+      <c r="B283" t="s">
+        <v>568</v>
+      </c>
+      <c r="C283" t="s">
+        <v>569</v>
+      </c>
+      <c r="D283" t="s">
+        <v>521</v>
+      </c>
+      <c r="E283" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="284" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A284">
+        <v>283</v>
+      </c>
+      <c r="B284" t="s">
+        <v>570</v>
+      </c>
+      <c r="C284" t="s">
+        <v>571</v>
+      </c>
+      <c r="D284" t="s">
+        <v>521</v>
+      </c>
+      <c r="E284" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="285" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A285">
+        <v>284</v>
+      </c>
+      <c r="B285" t="s">
+        <v>524</v>
+      </c>
+      <c r="C285" t="s">
+        <v>525</v>
+      </c>
+      <c r="D285" t="s">
+        <v>526</v>
+      </c>
+      <c r="E285" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="286" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A286">
+        <v>285</v>
+      </c>
+      <c r="B286" t="s">
+        <v>527</v>
+      </c>
+      <c r="C286" t="s">
+        <v>528</v>
+      </c>
+      <c r="D286" t="s">
+        <v>526</v>
+      </c>
+      <c r="E286" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="287" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A287">
+        <v>286</v>
+      </c>
+      <c r="B287" t="s">
+        <v>529</v>
+      </c>
+      <c r="C287" t="s">
+        <v>530</v>
+      </c>
+      <c r="D287" t="s">
+        <v>526</v>
+      </c>
+      <c r="E287" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="288" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A288">
+        <v>287</v>
+      </c>
+      <c r="B288" t="s">
+        <v>531</v>
+      </c>
+      <c r="C288" t="s">
+        <v>532</v>
+      </c>
+      <c r="D288" t="s">
+        <v>526</v>
+      </c>
+      <c r="E288" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="289" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A289">
+        <v>288</v>
+      </c>
+      <c r="B289" t="s">
+        <v>533</v>
+      </c>
+      <c r="C289" t="s">
+        <v>534</v>
+      </c>
+      <c r="D289" t="s">
+        <v>526</v>
+      </c>
+      <c r="E289" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="290" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A290">
+        <v>289</v>
+      </c>
+      <c r="B290" t="s">
+        <v>535</v>
+      </c>
+      <c r="C290" t="s">
+        <v>536</v>
+      </c>
+      <c r="D290" t="s">
+        <v>526</v>
+      </c>
+      <c r="E290" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="291" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A291">
+        <v>290</v>
+      </c>
+      <c r="B291" t="s">
+        <v>537</v>
+      </c>
+      <c r="C291" t="s">
+        <v>538</v>
+      </c>
+      <c r="D291" t="s">
+        <v>526</v>
+      </c>
+      <c r="E291" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="292" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A292">
+        <v>291</v>
+      </c>
+      <c r="B292" t="s">
+        <v>539</v>
+      </c>
+      <c r="C292" t="s">
+        <v>540</v>
+      </c>
+      <c r="D292" t="s">
+        <v>526</v>
+      </c>
+      <c r="E292" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="293" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A293">
+        <v>292</v>
+      </c>
+      <c r="B293" t="s">
+        <v>541</v>
+      </c>
+      <c r="C293" t="s">
+        <v>542</v>
+      </c>
+      <c r="D293" t="s">
+        <v>543</v>
+      </c>
+      <c r="E293" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="294" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A294">
+        <v>293</v>
+      </c>
+      <c r="B294" t="s">
+        <v>544</v>
+      </c>
+      <c r="C294" t="s">
+        <v>545</v>
+      </c>
+      <c r="D294" t="s">
+        <v>543</v>
+      </c>
+      <c r="E294" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="295" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A295">
+        <v>294</v>
+      </c>
+      <c r="B295" t="s">
+        <v>546</v>
+      </c>
+      <c r="C295" t="s">
+        <v>547</v>
+      </c>
+      <c r="D295" t="s">
+        <v>543</v>
+      </c>
+      <c r="E295" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="296" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A296">
+        <v>295</v>
+      </c>
+      <c r="B296" t="s">
+        <v>572</v>
+      </c>
+      <c r="C296" t="s">
+        <v>573</v>
+      </c>
+      <c r="D296" t="s">
+        <v>350</v>
+      </c>
+      <c r="E296" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="297" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A297">
+        <v>296</v>
+      </c>
+      <c r="B297" t="s">
+        <v>574</v>
+      </c>
+      <c r="C297" t="s">
+        <v>575</v>
+      </c>
+      <c r="D297" t="s">
+        <v>468</v>
+      </c>
+      <c r="E297" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="298" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A298">
+        <v>297</v>
+      </c>
+      <c r="B298" t="s">
         <v>576</v>
       </c>
-      <c r="C276" t="s">
+      <c r="C298" t="s">
         <v>577</v>
       </c>
-      <c r="D276" t="s">
+      <c r="D298" t="s">
         <v>578</v>
       </c>
-      <c r="E276" t="s">
+      <c r="E298" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="299" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A299">
+        <v>298</v>
+      </c>
+      <c r="B299" t="s">
+        <v>622</v>
+      </c>
+      <c r="C299" t="s">
+        <v>623</v>
+      </c>
+      <c r="D299" t="s">
+        <v>350</v>
+      </c>
+      <c r="E299" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="300" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A300">
+        <v>299</v>
+      </c>
+      <c r="B300" t="s">
+        <v>624</v>
+      </c>
+      <c r="C300" t="s">
+        <v>625</v>
+      </c>
+      <c r="D300" t="s">
+        <v>350</v>
+      </c>
+      <c r="E300" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="301" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A301">
+        <v>300</v>
+      </c>
+      <c r="B301" t="s">
+        <v>626</v>
+      </c>
+      <c r="C301" t="s">
+        <v>627</v>
+      </c>
+      <c r="D301" t="s">
+        <v>350</v>
+      </c>
+      <c r="E301" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="302" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A302">
+        <v>301</v>
+      </c>
+      <c r="B302" t="s">
+        <v>628</v>
+      </c>
+      <c r="C302" t="s">
+        <v>629</v>
+      </c>
+      <c r="D302" t="s">
+        <v>350</v>
+      </c>
+      <c r="E302" t="s">
         <v>488</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix duplicate PRN in roster
Kharade Sarthak Dasharath now has a distinct PRN (SELU126003),
resolving the SEFU126011 collision with Nade Ashutosh Abhijit
flagged in the previous roster update. Verified: no duplicate/
malformed PRNs, every group has a schedule, every program has a
registration room.
</commit_message>
<xml_diff>
--- a/Students Details.xlsx
+++ b/Students Details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Krishnendu.Jana\Desktop\MITVPU-Orientation-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F18D39F3-CE26-4DC5-A83D-B317BCE8B4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F629338-D28A-4974-AE82-6751770CD755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7991DB97-C80E-432A-B6FF-7E61A06C8A94}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="631">
   <si>
     <t>PRN</t>
   </si>
@@ -1703,9 +1703,6 @@
     <t>Kharade Sarthak Dasharath</t>
   </si>
   <si>
-    <t>SEFU126012</t>
-  </si>
-  <si>
     <t>Hulle Aadesh Abhay</t>
   </si>
   <si>
@@ -1751,9 +1748,6 @@
     <t>Holikatti Apoorva Subhashchandra</t>
   </si>
   <si>
-    <t>SDFU226004</t>
-  </si>
-  <si>
     <t>Rida Muzaffarhusain Maniyar</t>
   </si>
   <si>
@@ -1929,6 +1923,15 @@
   </si>
   <si>
     <t>Kshirsagar Aryan Amar</t>
+  </si>
+  <si>
+    <t>SELU126003</t>
+  </si>
+  <si>
+    <t>SELU126004</t>
+  </si>
+  <si>
+    <t>SDFU326009</t>
   </si>
 </sst>
 </file>
@@ -2931,10 +2934,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C37" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="D37" t="s">
         <v>4</v>
@@ -2948,10 +2951,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C38" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="D38" t="s">
         <v>4</v>
@@ -2965,10 +2968,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C39" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="D39" t="s">
         <v>84</v>
@@ -2982,10 +2985,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C40" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="D40" t="s">
         <v>84</v>
@@ -3563,7 +3566,7 @@
         <v>550</v>
       </c>
       <c r="C74" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="D74" t="s">
         <v>131</v>
@@ -3577,13 +3580,13 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>552</v>
+        <v>628</v>
       </c>
       <c r="C75" t="s">
         <v>553</v>
       </c>
       <c r="D75" t="s">
-        <v>131</v>
+        <v>443</v>
       </c>
       <c r="E75" t="s">
         <v>8</v>
@@ -3594,13 +3597,13 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>554</v>
+        <v>629</v>
       </c>
       <c r="C76" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="D76" t="s">
-        <v>131</v>
+        <v>443</v>
       </c>
       <c r="E76" t="s">
         <v>8</v>
@@ -4155,10 +4158,10 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
+        <v>555</v>
+      </c>
+      <c r="C109" t="s">
         <v>556</v>
-      </c>
-      <c r="C109" t="s">
-        <v>557</v>
       </c>
       <c r="D109" t="s">
         <v>150</v>
@@ -4172,10 +4175,10 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C110" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="D110" t="s">
         <v>150</v>
@@ -4189,10 +4192,10 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C111" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="D111" t="s">
         <v>150</v>
@@ -4206,10 +4209,10 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C112" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D112" t="s">
         <v>150</v>
@@ -4223,10 +4226,10 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="C113" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="D113" t="s">
         <v>150</v>
@@ -4240,10 +4243,10 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="C114" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="D114" t="s">
         <v>150</v>
@@ -4257,10 +4260,10 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="C115" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="D115" t="s">
         <v>150</v>
@@ -4274,13 +4277,13 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>213</v>
+        <v>559</v>
       </c>
       <c r="C116" t="s">
-        <v>214</v>
+        <v>560</v>
       </c>
       <c r="D116" t="s">
-        <v>215</v>
+        <v>4</v>
       </c>
       <c r="E116" t="s">
         <v>10</v>
@@ -4291,10 +4294,10 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C117" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D117" t="s">
         <v>215</v>
@@ -4308,10 +4311,10 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C118" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D118" t="s">
         <v>215</v>
@@ -4325,10 +4328,10 @@
         <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C119" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D119" t="s">
         <v>215</v>
@@ -4342,10 +4345,10 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C120" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D120" t="s">
         <v>215</v>
@@ -4359,10 +4362,10 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C121" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D121" t="s">
         <v>215</v>
@@ -4376,10 +4379,10 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C122" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D122" t="s">
         <v>215</v>
@@ -4393,10 +4396,10 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C123" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D123" t="s">
         <v>215</v>
@@ -4410,10 +4413,10 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C124" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D124" t="s">
         <v>215</v>
@@ -4427,10 +4430,10 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C125" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="D125" t="s">
         <v>215</v>
@@ -4444,10 +4447,10 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C126" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D126" t="s">
         <v>215</v>
@@ -4461,10 +4464,10 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C127" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D127" t="s">
         <v>215</v>
@@ -4478,10 +4481,10 @@
         <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C128" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D128" t="s">
         <v>215</v>
@@ -4495,10 +4498,10 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C129" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D129" t="s">
         <v>215</v>
@@ -4512,10 +4515,10 @@
         <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C130" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D130" t="s">
         <v>215</v>
@@ -4529,10 +4532,10 @@
         <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C131" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D131" t="s">
         <v>215</v>
@@ -4546,10 +4549,10 @@
         <v>131</v>
       </c>
       <c r="B132" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C132" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D132" t="s">
         <v>215</v>
@@ -4563,10 +4566,10 @@
         <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C133" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D133" t="s">
         <v>215</v>
@@ -4580,10 +4583,10 @@
         <v>133</v>
       </c>
       <c r="B134" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C134" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D134" t="s">
         <v>215</v>
@@ -4597,10 +4600,10 @@
         <v>134</v>
       </c>
       <c r="B135" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C135" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D135" t="s">
         <v>215</v>
@@ -4614,10 +4617,10 @@
         <v>135</v>
       </c>
       <c r="B136" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C136" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D136" t="s">
         <v>215</v>
@@ -4631,10 +4634,10 @@
         <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C137" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D137" t="s">
         <v>215</v>
@@ -4648,10 +4651,10 @@
         <v>137</v>
       </c>
       <c r="B138" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C138" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D138" t="s">
         <v>215</v>
@@ -4665,10 +4668,10 @@
         <v>138</v>
       </c>
       <c r="B139" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C139" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D139" t="s">
         <v>215</v>
@@ -4682,10 +4685,10 @@
         <v>139</v>
       </c>
       <c r="B140" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C140" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D140" t="s">
         <v>215</v>
@@ -4699,10 +4702,10 @@
         <v>140</v>
       </c>
       <c r="B141" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C141" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="D141" t="s">
         <v>215</v>
@@ -4716,10 +4719,10 @@
         <v>141</v>
       </c>
       <c r="B142" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C142" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D142" t="s">
         <v>215</v>
@@ -4733,10 +4736,10 @@
         <v>142</v>
       </c>
       <c r="B143" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C143" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D143" t="s">
         <v>215</v>
@@ -4750,10 +4753,10 @@
         <v>143</v>
       </c>
       <c r="B144" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C144" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D144" t="s">
         <v>215</v>
@@ -4767,10 +4770,10 @@
         <v>144</v>
       </c>
       <c r="B145" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C145" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="D145" t="s">
         <v>215</v>
@@ -4784,10 +4787,10 @@
         <v>145</v>
       </c>
       <c r="B146" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C146" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D146" t="s">
         <v>215</v>
@@ -4801,10 +4804,10 @@
         <v>146</v>
       </c>
       <c r="B147" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C147" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D147" t="s">
         <v>215</v>
@@ -4818,10 +4821,10 @@
         <v>147</v>
       </c>
       <c r="B148" t="s">
-        <v>558</v>
+        <v>276</v>
       </c>
       <c r="C148" t="s">
-        <v>559</v>
+        <v>277</v>
       </c>
       <c r="D148" t="s">
         <v>215</v>
@@ -4835,13 +4838,13 @@
         <v>148</v>
       </c>
       <c r="B149" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="C149" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="D149" t="s">
-        <v>4</v>
+        <v>215</v>
       </c>
       <c r="E149" t="s">
         <v>10</v>
@@ -4852,10 +4855,10 @@
         <v>149</v>
       </c>
       <c r="B150" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="C150" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="D150" t="s">
         <v>215</v>
@@ -4869,10 +4872,10 @@
         <v>150</v>
       </c>
       <c r="B151" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="C151" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="D151" t="s">
         <v>215</v>
@@ -4886,10 +4889,10 @@
         <v>151</v>
       </c>
       <c r="B152" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="C152" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="D152" t="s">
         <v>215</v>
@@ -4903,10 +4906,10 @@
         <v>152</v>
       </c>
       <c r="B153" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="C153" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="D153" t="s">
         <v>215</v>
@@ -4920,10 +4923,10 @@
         <v>153</v>
       </c>
       <c r="B154" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="C154" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="D154" t="s">
         <v>215</v>
@@ -6076,10 +6079,10 @@
         <v>221</v>
       </c>
       <c r="B222" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="C222" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="D222" t="s">
         <v>3</v>
@@ -6093,13 +6096,13 @@
         <v>222</v>
       </c>
       <c r="B223" t="s">
+        <v>552</v>
+      </c>
+      <c r="C223" t="s">
         <v>611</v>
       </c>
-      <c r="C223" t="s">
-        <v>612</v>
-      </c>
       <c r="D223" t="s">
-        <v>443</v>
+        <v>131</v>
       </c>
       <c r="E223" t="s">
         <v>351</v>
@@ -6110,13 +6113,13 @@
         <v>223</v>
       </c>
       <c r="B224" t="s">
-        <v>552</v>
+        <v>609</v>
       </c>
       <c r="C224" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="D224" t="s">
-        <v>131</v>
+        <v>443</v>
       </c>
       <c r="E224" t="s">
         <v>351</v>
@@ -6127,13 +6130,13 @@
         <v>224</v>
       </c>
       <c r="B225" t="s">
-        <v>414</v>
+        <v>466</v>
       </c>
       <c r="C225" t="s">
-        <v>415</v>
+        <v>467</v>
       </c>
       <c r="D225" t="s">
-        <v>350</v>
+        <v>468</v>
       </c>
       <c r="E225" t="s">
         <v>416</v>
@@ -6144,13 +6147,13 @@
         <v>225</v>
       </c>
       <c r="B226" t="s">
-        <v>417</v>
+        <v>469</v>
       </c>
       <c r="C226" t="s">
-        <v>418</v>
+        <v>470</v>
       </c>
       <c r="D226" t="s">
-        <v>350</v>
+        <v>468</v>
       </c>
       <c r="E226" t="s">
         <v>416</v>
@@ -6161,13 +6164,13 @@
         <v>226</v>
       </c>
       <c r="B227" t="s">
-        <v>419</v>
+        <v>471</v>
       </c>
       <c r="C227" t="s">
-        <v>420</v>
+        <v>472</v>
       </c>
       <c r="D227" t="s">
-        <v>350</v>
+        <v>468</v>
       </c>
       <c r="E227" t="s">
         <v>416</v>
@@ -6178,13 +6181,13 @@
         <v>227</v>
       </c>
       <c r="B228" t="s">
-        <v>421</v>
+        <v>473</v>
       </c>
       <c r="C228" t="s">
-        <v>422</v>
+        <v>474</v>
       </c>
       <c r="D228" t="s">
-        <v>350</v>
+        <v>468</v>
       </c>
       <c r="E228" t="s">
         <v>416</v>
@@ -6195,13 +6198,13 @@
         <v>228</v>
       </c>
       <c r="B229" t="s">
-        <v>423</v>
+        <v>475</v>
       </c>
       <c r="C229" t="s">
-        <v>424</v>
+        <v>476</v>
       </c>
       <c r="D229" t="s">
-        <v>350</v>
+        <v>468</v>
       </c>
       <c r="E229" t="s">
         <v>416</v>
@@ -6212,13 +6215,13 @@
         <v>229</v>
       </c>
       <c r="B230" t="s">
-        <v>425</v>
+        <v>477</v>
       </c>
       <c r="C230" t="s">
-        <v>426</v>
+        <v>478</v>
       </c>
       <c r="D230" t="s">
-        <v>350</v>
+        <v>468</v>
       </c>
       <c r="E230" t="s">
         <v>416</v>
@@ -6229,13 +6232,13 @@
         <v>230</v>
       </c>
       <c r="B231" t="s">
-        <v>427</v>
+        <v>479</v>
       </c>
       <c r="C231" t="s">
-        <v>428</v>
+        <v>480</v>
       </c>
       <c r="D231" t="s">
-        <v>350</v>
+        <v>468</v>
       </c>
       <c r="E231" t="s">
         <v>416</v>
@@ -6246,13 +6249,13 @@
         <v>231</v>
       </c>
       <c r="B232" t="s">
-        <v>429</v>
+        <v>481</v>
       </c>
       <c r="C232" t="s">
-        <v>430</v>
+        <v>482</v>
       </c>
       <c r="D232" t="s">
-        <v>350</v>
+        <v>468</v>
       </c>
       <c r="E232" t="s">
         <v>416</v>
@@ -6263,13 +6266,13 @@
         <v>232</v>
       </c>
       <c r="B233" t="s">
-        <v>431</v>
+        <v>483</v>
       </c>
       <c r="C233" t="s">
-        <v>432</v>
+        <v>484</v>
       </c>
       <c r="D233" t="s">
-        <v>350</v>
+        <v>468</v>
       </c>
       <c r="E233" t="s">
         <v>416</v>
@@ -6280,13 +6283,13 @@
         <v>233</v>
       </c>
       <c r="B234" t="s">
-        <v>433</v>
+        <v>612</v>
       </c>
       <c r="C234" t="s">
-        <v>434</v>
+        <v>613</v>
       </c>
       <c r="D234" t="s">
-        <v>350</v>
+        <v>468</v>
       </c>
       <c r="E234" t="s">
         <v>416</v>
@@ -6297,13 +6300,13 @@
         <v>234</v>
       </c>
       <c r="B235" t="s">
-        <v>435</v>
+        <v>616</v>
       </c>
       <c r="C235" t="s">
-        <v>436</v>
+        <v>617</v>
       </c>
       <c r="D235" t="s">
-        <v>350</v>
+        <v>487</v>
       </c>
       <c r="E235" t="s">
         <v>416</v>
@@ -6314,13 +6317,13 @@
         <v>235</v>
       </c>
       <c r="B236" t="s">
-        <v>437</v>
+        <v>618</v>
       </c>
       <c r="C236" t="s">
-        <v>438</v>
+        <v>619</v>
       </c>
       <c r="D236" t="s">
-        <v>350</v>
+        <v>487</v>
       </c>
       <c r="E236" t="s">
         <v>416</v>
@@ -6331,10 +6334,10 @@
         <v>236</v>
       </c>
       <c r="B237" t="s">
-        <v>439</v>
+        <v>414</v>
       </c>
       <c r="C237" t="s">
-        <v>440</v>
+        <v>415</v>
       </c>
       <c r="D237" t="s">
         <v>350</v>
@@ -6348,13 +6351,13 @@
         <v>237</v>
       </c>
       <c r="B238" t="s">
-        <v>441</v>
+        <v>417</v>
       </c>
       <c r="C238" t="s">
-        <v>442</v>
+        <v>418</v>
       </c>
       <c r="D238" t="s">
-        <v>443</v>
+        <v>350</v>
       </c>
       <c r="E238" t="s">
         <v>416</v>
@@ -6365,13 +6368,13 @@
         <v>238</v>
       </c>
       <c r="B239" t="s">
-        <v>444</v>
+        <v>419</v>
       </c>
       <c r="C239" t="s">
-        <v>445</v>
+        <v>420</v>
       </c>
       <c r="D239" t="s">
-        <v>443</v>
+        <v>350</v>
       </c>
       <c r="E239" t="s">
         <v>416</v>
@@ -6382,13 +6385,13 @@
         <v>239</v>
       </c>
       <c r="B240" t="s">
-        <v>446</v>
+        <v>421</v>
       </c>
       <c r="C240" t="s">
-        <v>447</v>
+        <v>422</v>
       </c>
       <c r="D240" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E240" t="s">
         <v>416</v>
@@ -6399,13 +6402,13 @@
         <v>240</v>
       </c>
       <c r="B241" t="s">
-        <v>448</v>
+        <v>423</v>
       </c>
       <c r="C241" t="s">
-        <v>449</v>
+        <v>424</v>
       </c>
       <c r="D241" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E241" t="s">
         <v>416</v>
@@ -6416,13 +6419,13 @@
         <v>241</v>
       </c>
       <c r="B242" t="s">
-        <v>450</v>
+        <v>425</v>
       </c>
       <c r="C242" t="s">
-        <v>451</v>
+        <v>426</v>
       </c>
       <c r="D242" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E242" t="s">
         <v>416</v>
@@ -6433,13 +6436,13 @@
         <v>242</v>
       </c>
       <c r="B243" t="s">
-        <v>452</v>
+        <v>427</v>
       </c>
       <c r="C243" t="s">
-        <v>453</v>
+        <v>428</v>
       </c>
       <c r="D243" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E243" t="s">
         <v>416</v>
@@ -6450,13 +6453,13 @@
         <v>243</v>
       </c>
       <c r="B244" t="s">
-        <v>454</v>
+        <v>429</v>
       </c>
       <c r="C244" t="s">
-        <v>455</v>
+        <v>430</v>
       </c>
       <c r="D244" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E244" t="s">
         <v>416</v>
@@ -6467,13 +6470,13 @@
         <v>244</v>
       </c>
       <c r="B245" t="s">
-        <v>456</v>
+        <v>431</v>
       </c>
       <c r="C245" t="s">
-        <v>457</v>
+        <v>432</v>
       </c>
       <c r="D245" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E245" t="s">
         <v>416</v>
@@ -6484,13 +6487,13 @@
         <v>245</v>
       </c>
       <c r="B246" t="s">
-        <v>458</v>
+        <v>433</v>
       </c>
       <c r="C246" t="s">
-        <v>459</v>
+        <v>434</v>
       </c>
       <c r="D246" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E246" t="s">
         <v>416</v>
@@ -6501,13 +6504,13 @@
         <v>246</v>
       </c>
       <c r="B247" t="s">
-        <v>460</v>
+        <v>435</v>
       </c>
       <c r="C247" t="s">
-        <v>461</v>
+        <v>436</v>
       </c>
       <c r="D247" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E247" t="s">
         <v>416</v>
@@ -6518,13 +6521,13 @@
         <v>247</v>
       </c>
       <c r="B248" t="s">
-        <v>462</v>
+        <v>437</v>
       </c>
       <c r="C248" t="s">
-        <v>463</v>
+        <v>438</v>
       </c>
       <c r="D248" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E248" t="s">
         <v>416</v>
@@ -6535,13 +6538,13 @@
         <v>248</v>
       </c>
       <c r="B249" t="s">
-        <v>464</v>
+        <v>439</v>
       </c>
       <c r="C249" t="s">
-        <v>465</v>
+        <v>440</v>
       </c>
       <c r="D249" t="s">
-        <v>3</v>
+        <v>350</v>
       </c>
       <c r="E249" t="s">
         <v>416</v>
@@ -6552,10 +6555,10 @@
         <v>249</v>
       </c>
       <c r="B250" t="s">
-        <v>562</v>
+        <v>446</v>
       </c>
       <c r="C250" t="s">
-        <v>563</v>
+        <v>447</v>
       </c>
       <c r="D250" t="s">
         <v>3</v>
@@ -6569,13 +6572,13 @@
         <v>250</v>
       </c>
       <c r="B251" t="s">
-        <v>466</v>
+        <v>448</v>
       </c>
       <c r="C251" t="s">
-        <v>467</v>
+        <v>449</v>
       </c>
       <c r="D251" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E251" t="s">
         <v>416</v>
@@ -6586,13 +6589,13 @@
         <v>251</v>
       </c>
       <c r="B252" t="s">
-        <v>469</v>
+        <v>450</v>
       </c>
       <c r="C252" t="s">
-        <v>470</v>
+        <v>451</v>
       </c>
       <c r="D252" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E252" t="s">
         <v>416</v>
@@ -6603,13 +6606,13 @@
         <v>252</v>
       </c>
       <c r="B253" t="s">
-        <v>471</v>
+        <v>452</v>
       </c>
       <c r="C253" t="s">
-        <v>472</v>
+        <v>453</v>
       </c>
       <c r="D253" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E253" t="s">
         <v>416</v>
@@ -6620,13 +6623,13 @@
         <v>253</v>
       </c>
       <c r="B254" t="s">
-        <v>473</v>
+        <v>454</v>
       </c>
       <c r="C254" t="s">
-        <v>474</v>
+        <v>455</v>
       </c>
       <c r="D254" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E254" t="s">
         <v>416</v>
@@ -6637,13 +6640,13 @@
         <v>254</v>
       </c>
       <c r="B255" t="s">
-        <v>475</v>
+        <v>456</v>
       </c>
       <c r="C255" t="s">
-        <v>476</v>
+        <v>457</v>
       </c>
       <c r="D255" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E255" t="s">
         <v>416</v>
@@ -6654,13 +6657,13 @@
         <v>255</v>
       </c>
       <c r="B256" t="s">
-        <v>477</v>
+        <v>458</v>
       </c>
       <c r="C256" t="s">
-        <v>478</v>
+        <v>459</v>
       </c>
       <c r="D256" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E256" t="s">
         <v>416</v>
@@ -6671,13 +6674,13 @@
         <v>256</v>
       </c>
       <c r="B257" t="s">
-        <v>479</v>
+        <v>460</v>
       </c>
       <c r="C257" t="s">
-        <v>480</v>
+        <v>461</v>
       </c>
       <c r="D257" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E257" t="s">
         <v>416</v>
@@ -6688,13 +6691,13 @@
         <v>257</v>
       </c>
       <c r="B258" t="s">
-        <v>481</v>
+        <v>462</v>
       </c>
       <c r="C258" t="s">
-        <v>482</v>
+        <v>463</v>
       </c>
       <c r="D258" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E258" t="s">
         <v>416</v>
@@ -6705,13 +6708,13 @@
         <v>258</v>
       </c>
       <c r="B259" t="s">
-        <v>483</v>
+        <v>464</v>
       </c>
       <c r="C259" t="s">
-        <v>484</v>
+        <v>465</v>
       </c>
       <c r="D259" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E259" t="s">
         <v>416</v>
@@ -6722,13 +6725,13 @@
         <v>259</v>
       </c>
       <c r="B260" t="s">
-        <v>614</v>
+        <v>561</v>
       </c>
       <c r="C260" t="s">
-        <v>615</v>
+        <v>562</v>
       </c>
       <c r="D260" t="s">
-        <v>468</v>
+        <v>3</v>
       </c>
       <c r="E260" t="s">
         <v>416</v>
@@ -6739,13 +6742,13 @@
         <v>260</v>
       </c>
       <c r="B261" t="s">
-        <v>616</v>
+        <v>441</v>
       </c>
       <c r="C261" t="s">
-        <v>617</v>
+        <v>442</v>
       </c>
       <c r="D261" t="s">
-        <v>543</v>
+        <v>443</v>
       </c>
       <c r="E261" t="s">
         <v>416</v>
@@ -6756,13 +6759,13 @@
         <v>261</v>
       </c>
       <c r="B262" t="s">
-        <v>618</v>
+        <v>444</v>
       </c>
       <c r="C262" t="s">
-        <v>619</v>
+        <v>445</v>
       </c>
       <c r="D262" t="s">
-        <v>487</v>
+        <v>443</v>
       </c>
       <c r="E262" t="s">
         <v>416</v>
@@ -6773,13 +6776,13 @@
         <v>262</v>
       </c>
       <c r="B263" t="s">
-        <v>620</v>
+        <v>614</v>
       </c>
       <c r="C263" t="s">
-        <v>621</v>
+        <v>615</v>
       </c>
       <c r="D263" t="s">
-        <v>487</v>
+        <v>543</v>
       </c>
       <c r="E263" t="s">
         <v>416</v>
@@ -6790,13 +6793,13 @@
         <v>263</v>
       </c>
       <c r="B264" t="s">
-        <v>485</v>
+        <v>572</v>
       </c>
       <c r="C264" t="s">
-        <v>486</v>
+        <v>573</v>
       </c>
       <c r="D264" t="s">
-        <v>487</v>
+        <v>468</v>
       </c>
       <c r="E264" t="s">
         <v>488</v>
@@ -6807,10 +6810,10 @@
         <v>264</v>
       </c>
       <c r="B265" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="C265" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="D265" t="s">
         <v>487</v>
@@ -6824,10 +6827,10 @@
         <v>265</v>
       </c>
       <c r="B266" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="C266" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D266" t="s">
         <v>487</v>
@@ -6841,10 +6844,10 @@
         <v>266</v>
       </c>
       <c r="B267" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="C267" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="D267" t="s">
         <v>487</v>
@@ -6858,10 +6861,10 @@
         <v>267</v>
       </c>
       <c r="B268" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="C268" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D268" t="s">
         <v>487</v>
@@ -6875,10 +6878,10 @@
         <v>268</v>
       </c>
       <c r="B269" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="C269" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="D269" t="s">
         <v>487</v>
@@ -6892,10 +6895,10 @@
         <v>269</v>
       </c>
       <c r="B270" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C270" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="D270" t="s">
         <v>487</v>
@@ -6909,10 +6912,10 @@
         <v>270</v>
       </c>
       <c r="B271" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C271" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D271" t="s">
         <v>487</v>
@@ -6926,10 +6929,10 @@
         <v>271</v>
       </c>
       <c r="B272" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C272" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D272" t="s">
         <v>487</v>
@@ -6943,10 +6946,10 @@
         <v>272</v>
       </c>
       <c r="B273" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C273" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D273" t="s">
         <v>487</v>
@@ -6960,10 +6963,10 @@
         <v>273</v>
       </c>
       <c r="B274" t="s">
-        <v>564</v>
+        <v>505</v>
       </c>
       <c r="C274" t="s">
-        <v>565</v>
+        <v>506</v>
       </c>
       <c r="D274" t="s">
         <v>487</v>
@@ -6977,10 +6980,10 @@
         <v>274</v>
       </c>
       <c r="B275" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="C275" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="D275" t="s">
         <v>487</v>
@@ -6994,13 +6997,13 @@
         <v>275</v>
       </c>
       <c r="B276" t="s">
-        <v>507</v>
+        <v>565</v>
       </c>
       <c r="C276" t="s">
-        <v>508</v>
+        <v>566</v>
       </c>
       <c r="D276" t="s">
-        <v>509</v>
+        <v>487</v>
       </c>
       <c r="E276" t="s">
         <v>488</v>
@@ -7011,13 +7014,13 @@
         <v>276</v>
       </c>
       <c r="B277" t="s">
-        <v>510</v>
+        <v>570</v>
       </c>
       <c r="C277" t="s">
-        <v>511</v>
+        <v>571</v>
       </c>
       <c r="D277" t="s">
-        <v>509</v>
+        <v>350</v>
       </c>
       <c r="E277" t="s">
         <v>488</v>
@@ -7028,13 +7031,13 @@
         <v>277</v>
       </c>
       <c r="B278" t="s">
-        <v>512</v>
+        <v>620</v>
       </c>
       <c r="C278" t="s">
-        <v>513</v>
+        <v>621</v>
       </c>
       <c r="D278" t="s">
-        <v>514</v>
+        <v>350</v>
       </c>
       <c r="E278" t="s">
         <v>488</v>
@@ -7045,13 +7048,13 @@
         <v>278</v>
       </c>
       <c r="B279" t="s">
-        <v>515</v>
+        <v>622</v>
       </c>
       <c r="C279" t="s">
-        <v>516</v>
+        <v>623</v>
       </c>
       <c r="D279" t="s">
-        <v>514</v>
+        <v>350</v>
       </c>
       <c r="E279" t="s">
         <v>488</v>
@@ -7062,13 +7065,13 @@
         <v>279</v>
       </c>
       <c r="B280" t="s">
-        <v>517</v>
+        <v>624</v>
       </c>
       <c r="C280" t="s">
-        <v>518</v>
+        <v>625</v>
       </c>
       <c r="D280" t="s">
-        <v>514</v>
+        <v>350</v>
       </c>
       <c r="E280" t="s">
         <v>488</v>
@@ -7079,13 +7082,13 @@
         <v>280</v>
       </c>
       <c r="B281" t="s">
-        <v>519</v>
+        <v>626</v>
       </c>
       <c r="C281" t="s">
-        <v>520</v>
+        <v>627</v>
       </c>
       <c r="D281" t="s">
-        <v>521</v>
+        <v>350</v>
       </c>
       <c r="E281" t="s">
         <v>488</v>
@@ -7096,13 +7099,13 @@
         <v>281</v>
       </c>
       <c r="B282" t="s">
-        <v>522</v>
+        <v>507</v>
       </c>
       <c r="C282" t="s">
-        <v>523</v>
+        <v>508</v>
       </c>
       <c r="D282" t="s">
-        <v>521</v>
+        <v>509</v>
       </c>
       <c r="E282" t="s">
         <v>488</v>
@@ -7113,13 +7116,13 @@
         <v>282</v>
       </c>
       <c r="B283" t="s">
-        <v>568</v>
+        <v>510</v>
       </c>
       <c r="C283" t="s">
-        <v>569</v>
+        <v>511</v>
       </c>
       <c r="D283" t="s">
-        <v>521</v>
+        <v>509</v>
       </c>
       <c r="E283" t="s">
         <v>488</v>
@@ -7130,13 +7133,13 @@
         <v>283</v>
       </c>
       <c r="B284" t="s">
-        <v>570</v>
+        <v>512</v>
       </c>
       <c r="C284" t="s">
-        <v>571</v>
+        <v>513</v>
       </c>
       <c r="D284" t="s">
-        <v>521</v>
+        <v>514</v>
       </c>
       <c r="E284" t="s">
         <v>488</v>
@@ -7147,13 +7150,13 @@
         <v>284</v>
       </c>
       <c r="B285" t="s">
-        <v>524</v>
+        <v>515</v>
       </c>
       <c r="C285" t="s">
-        <v>525</v>
+        <v>516</v>
       </c>
       <c r="D285" t="s">
-        <v>526</v>
+        <v>514</v>
       </c>
       <c r="E285" t="s">
         <v>488</v>
@@ -7164,13 +7167,13 @@
         <v>285</v>
       </c>
       <c r="B286" t="s">
-        <v>527</v>
+        <v>517</v>
       </c>
       <c r="C286" t="s">
-        <v>528</v>
+        <v>518</v>
       </c>
       <c r="D286" t="s">
-        <v>526</v>
+        <v>514</v>
       </c>
       <c r="E286" t="s">
         <v>488</v>
@@ -7181,13 +7184,13 @@
         <v>286</v>
       </c>
       <c r="B287" t="s">
-        <v>529</v>
+        <v>519</v>
       </c>
       <c r="C287" t="s">
-        <v>530</v>
+        <v>520</v>
       </c>
       <c r="D287" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="E287" t="s">
         <v>488</v>
@@ -7198,13 +7201,13 @@
         <v>287</v>
       </c>
       <c r="B288" t="s">
-        <v>531</v>
+        <v>522</v>
       </c>
       <c r="C288" t="s">
-        <v>532</v>
+        <v>523</v>
       </c>
       <c r="D288" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="E288" t="s">
         <v>488</v>
@@ -7215,13 +7218,13 @@
         <v>288</v>
       </c>
       <c r="B289" t="s">
-        <v>533</v>
+        <v>567</v>
       </c>
       <c r="C289" t="s">
-        <v>534</v>
+        <v>568</v>
       </c>
       <c r="D289" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="E289" t="s">
         <v>488</v>
@@ -7232,10 +7235,10 @@
         <v>289</v>
       </c>
       <c r="B290" t="s">
-        <v>535</v>
+        <v>524</v>
       </c>
       <c r="C290" t="s">
-        <v>536</v>
+        <v>525</v>
       </c>
       <c r="D290" t="s">
         <v>526</v>
@@ -7249,10 +7252,10 @@
         <v>290</v>
       </c>
       <c r="B291" t="s">
-        <v>537</v>
+        <v>527</v>
       </c>
       <c r="C291" t="s">
-        <v>538</v>
+        <v>528</v>
       </c>
       <c r="D291" t="s">
         <v>526</v>
@@ -7266,10 +7269,10 @@
         <v>291</v>
       </c>
       <c r="B292" t="s">
-        <v>539</v>
+        <v>529</v>
       </c>
       <c r="C292" t="s">
-        <v>540</v>
+        <v>530</v>
       </c>
       <c r="D292" t="s">
         <v>526</v>
@@ -7283,13 +7286,13 @@
         <v>292</v>
       </c>
       <c r="B293" t="s">
-        <v>541</v>
+        <v>531</v>
       </c>
       <c r="C293" t="s">
-        <v>542</v>
+        <v>532</v>
       </c>
       <c r="D293" t="s">
-        <v>543</v>
+        <v>526</v>
       </c>
       <c r="E293" t="s">
         <v>488</v>
@@ -7300,13 +7303,13 @@
         <v>293</v>
       </c>
       <c r="B294" t="s">
-        <v>544</v>
+        <v>533</v>
       </c>
       <c r="C294" t="s">
-        <v>545</v>
+        <v>534</v>
       </c>
       <c r="D294" t="s">
-        <v>543</v>
+        <v>526</v>
       </c>
       <c r="E294" t="s">
         <v>488</v>
@@ -7317,13 +7320,13 @@
         <v>294</v>
       </c>
       <c r="B295" t="s">
-        <v>546</v>
+        <v>535</v>
       </c>
       <c r="C295" t="s">
-        <v>547</v>
+        <v>536</v>
       </c>
       <c r="D295" t="s">
-        <v>543</v>
+        <v>526</v>
       </c>
       <c r="E295" t="s">
         <v>488</v>
@@ -7334,13 +7337,13 @@
         <v>295</v>
       </c>
       <c r="B296" t="s">
-        <v>572</v>
+        <v>537</v>
       </c>
       <c r="C296" t="s">
-        <v>573</v>
+        <v>538</v>
       </c>
       <c r="D296" t="s">
-        <v>350</v>
+        <v>526</v>
       </c>
       <c r="E296" t="s">
         <v>488</v>
@@ -7351,13 +7354,13 @@
         <v>296</v>
       </c>
       <c r="B297" t="s">
-        <v>574</v>
+        <v>539</v>
       </c>
       <c r="C297" t="s">
-        <v>575</v>
+        <v>540</v>
       </c>
       <c r="D297" t="s">
-        <v>468</v>
+        <v>526</v>
       </c>
       <c r="E297" t="s">
         <v>488</v>
@@ -7368,13 +7371,13 @@
         <v>297</v>
       </c>
       <c r="B298" t="s">
-        <v>576</v>
+        <v>630</v>
       </c>
       <c r="C298" t="s">
-        <v>577</v>
+        <v>569</v>
       </c>
       <c r="D298" t="s">
-        <v>578</v>
+        <v>526</v>
       </c>
       <c r="E298" t="s">
         <v>488</v>
@@ -7385,13 +7388,13 @@
         <v>298</v>
       </c>
       <c r="B299" t="s">
-        <v>622</v>
+        <v>541</v>
       </c>
       <c r="C299" t="s">
-        <v>623</v>
+        <v>542</v>
       </c>
       <c r="D299" t="s">
-        <v>350</v>
+        <v>543</v>
       </c>
       <c r="E299" t="s">
         <v>488</v>
@@ -7402,13 +7405,13 @@
         <v>299</v>
       </c>
       <c r="B300" t="s">
-        <v>624</v>
+        <v>544</v>
       </c>
       <c r="C300" t="s">
-        <v>625</v>
+        <v>545</v>
       </c>
       <c r="D300" t="s">
-        <v>350</v>
+        <v>543</v>
       </c>
       <c r="E300" t="s">
         <v>488</v>
@@ -7419,13 +7422,13 @@
         <v>300</v>
       </c>
       <c r="B301" t="s">
-        <v>626</v>
+        <v>546</v>
       </c>
       <c r="C301" t="s">
-        <v>627</v>
+        <v>547</v>
       </c>
       <c r="D301" t="s">
-        <v>350</v>
+        <v>543</v>
       </c>
       <c r="E301" t="s">
         <v>488</v>
@@ -7436,13 +7439,13 @@
         <v>301</v>
       </c>
       <c r="B302" t="s">
-        <v>628</v>
+        <v>574</v>
       </c>
       <c r="C302" t="s">
-        <v>629</v>
+        <v>575</v>
       </c>
       <c r="D302" t="s">
-        <v>350</v>
+        <v>576</v>
       </c>
       <c r="E302" t="s">
         <v>488</v>

</xml_diff>